<commit_message>
DB + Redis foundation + real health probes + baseline migration
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,12 +495,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/health/db</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Readiness probe</t>
+          <t>Database readiness probe</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -515,6 +515,72 @@
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
         <is>
           <t>200</t>
         </is>

</xml_diff>

<commit_message>
users + JWT auth + RBAC + rate limit
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,22 +457,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/auth/login</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>auth</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -480,43 +480,47 @@
           <t>public</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>LoginRequest</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/api/v1/auth/logout</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Logout</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>auth</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204</t>
         </is>
       </c>
     </row>
@@ -528,22 +532,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/api/v1/auth/me</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Me</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>auth</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -556,31 +560,204 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>/api/v1/auth/refresh</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Refresh</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>auth</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>RefreshRequest</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>/api/v1/auth/register</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>auth</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>RegisterRequest</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>201, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>/health</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Liveness probe</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>/health/db</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Database readiness probe</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>/health/redis</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Redis readiness probe</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>health</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -597,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -617,6 +794,159 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AuthTokens</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>access_token, refresh_token, token_type, expires_in</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HTTPValidationError</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>LoginRequest</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>email, password</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LoginResponse</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>user, tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RefreshRequest</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>refresh_token</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RegisterRequest</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>email, password</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RegisterResponse</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>user, message</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ValidationError</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>loc, msg, type, input, ctx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
users API + profile + consent + soft-delete + optimistic lock
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -634,27 +634,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -672,22 +672,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>My profile</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -700,33 +700,37 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Update my profile</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>public</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -738,26 +742,261 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>/api/v1/users/me/consent</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Grant consent</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>201, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>/api/v1/users/me/consent/{channel}</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Revoke Consent</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>204, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Public profile</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>/health</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Liveness probe</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>/health/db</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Database readiness probe</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -774,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -814,7 +1053,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HTTPValidationError</t>
+          <t>ConsentGrantRequest</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -824,14 +1063,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>channel</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>ConsentList</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -841,14 +1080,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>consents</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LoginResponse</t>
+          <t>ConsentRecord</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -858,14 +1097,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>channel, granted, granted_at, revoked_at</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>DeleteMeResponse</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -875,14 +1114,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>message, hard_delete_after</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>HTTPValidationError</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -892,14 +1131,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>detail</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>LoginRequest</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -909,14 +1148,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>LoginResponse</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -926,22 +1165,141 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>user, tokens</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>ProfilePublic</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ProfileSelf</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RefreshRequest</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>refresh_token</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RegisterRequest</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>email, password</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RegisterResponse</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>user, message</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
Follows (social graph) + block/mute + FOLLOWERS visibility
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -639,17 +639,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/blocks/{user_id}</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Unblock</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -660,29 +660,29 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/blocks/{user_id}</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>My profile</t>
+          <t>Block</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -693,29 +693,29 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Update my profile</t>
+          <t>Unfollow a user (idempotent)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -723,36 +723,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>ProfileUpdate</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>Follow a user (idempotent)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -763,29 +759,29 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Grant consent</t>
+          <t>Unmute</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -793,36 +789,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>ConsentGrantRequest</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Mute</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -840,17 +832,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Public profile</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -866,7 +858,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -878,22 +870,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -906,33 +898,37 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>public</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -944,22 +940,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -972,31 +968,365 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>/api/v1/users/me/consent</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Grant Consent</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>201, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>/api/v1/users/me/consent/{channel}</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Revoke Consent</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>204, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Get Profile</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/follow-status</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Status Endpoint</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/followers</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Followers</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/following</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Following</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>/health</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Liveness probe</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>/health/db</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Database readiness probe</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
         <is>
           <t>/health/redis</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Redis readiness probe</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>health</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -1013,7 +1343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1121,7 +1451,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HTTPValidationError</t>
+          <t>FollowCounts</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1131,14 +1461,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>followers, following</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>FollowListPage</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1148,14 +1478,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LoginResponse</t>
+          <t>FollowStatus</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1165,14 +1495,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>FollowUserView</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1182,14 +1512,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>user_id, display_name, avatar_url, followed_at</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>HTTPValidationError</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1199,14 +1529,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>detail</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>LoginRequest</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1216,14 +1546,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>LoginResponse</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1233,14 +1563,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>user, tokens</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>ProfilePublic</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1250,14 +1580,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>ProfileSelf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1267,14 +1597,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1284,22 +1614,90 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>RefreshRequest</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>refresh_token</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>RegisterRequest</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>email, password</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>RegisterResponse</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>user, message</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
posts + comments + likes with cursor pagination + counter caches
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -705,17 +705,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/comments/{comment_id}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Unfollow a user (idempotent)</t>
+          <t>Delete Comment</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -733,22 +733,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/comments/{comment_id}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Follow a user (idempotent)</t>
+          <t>Update Comment</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -756,10 +756,14 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>CommentUpdate</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -771,12 +775,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Unmute</t>
+          <t>Unfollow a user (idempotent)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -804,12 +808,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mute</t>
+          <t>Follow a user (idempotent)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -837,17 +841,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Unlike</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -858,29 +862,29 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Like</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -891,29 +895,29 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>List Likers</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -921,11 +925,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>ProfileUpdate</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -935,22 +935,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>Unmute</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -961,7 +961,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -973,17 +973,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>Mute</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -991,36 +991,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>ConsentGrantRequest</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/posts</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Create Post</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1028,10 +1024,14 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PostCreate</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -1043,17 +1043,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/posts/by-author/{author_id}</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>List By Author</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1071,22 +1071,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Delete Post</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1097,7 +1097,7 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1109,17 +1109,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>Get Post</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1137,22 +1137,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Update Post</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1160,7 +1160,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>PostUpdate</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1175,17 +1179,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>List Comments</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1203,60 +1207,64 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Create Comment</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>public</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>CommentCreate</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -1274,22 +1282,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -1302,31 +1310,435 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>/api/v1/users/me</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Update Me</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>/api/v1/users/me/consent</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>List Consents</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>/api/v1/users/me/consent</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Grant Consent</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>201, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>/api/v1/users/me/consent/{channel}</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Revoke Consent</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>204, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Get Profile</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/follow-status</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Status Endpoint</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/followers</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Followers</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/following</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Following</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>/health</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Liveness probe</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>/health/db</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Database readiness probe</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
         <is>
           <t>/health/redis</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Redis readiness probe</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>health</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -1343,7 +1755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1383,7 +1795,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ConsentGrantRequest</t>
+          <t>CommentCreate</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1393,14 +1805,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>body, parent_id</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ConsentList</t>
+          <t>CommentPage</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1410,14 +1822,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>consents</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ConsentRecord</t>
+          <t>CommentUpdate</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1427,14 +1839,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>channel, granted, granted_at, revoked_at</t>
+          <t>body, version</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DeleteMeResponse</t>
+          <t>CommentView</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1444,14 +1856,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>message, hard_delete_after</t>
+          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at, is_liked_by_me, is_edited, replies</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FollowCounts</t>
+          <t>ConsentGrantRequest</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1461,14 +1873,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>followers, following</t>
+          <t>channel</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FollowListPage</t>
+          <t>ConsentList</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1478,14 +1890,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>consents</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FollowStatus</t>
+          <t>ConsentRecord</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1495,14 +1907,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
+          <t>channel, granted, granted_at, revoked_at</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FollowUserView</t>
+          <t>DeleteMeResponse</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1512,14 +1924,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url, followed_at</t>
+          <t>message, hard_delete_after</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HTTPValidationError</t>
+          <t>FollowCounts</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1529,14 +1941,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>followers, following</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>FollowListPage</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1546,14 +1958,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LoginResponse</t>
+          <t>FollowStatus</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1563,14 +1975,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>FollowUserView</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1580,14 +1992,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>user_id, display_name, avatar_url, followed_at</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>HTTPValidationError</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1597,14 +2009,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>detail</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>LikeUser</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1614,14 +2026,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>user_id, display_name, avatar_url</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>LikeUserPage</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1631,14 +2043,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>LoginRequest</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1655,7 +2067,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>LoginResponse</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1665,14 +2077,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>user, tokens</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1682,22 +2094,192 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>body, visibility</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>PostPage</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>items, next_cursor</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PostUpdate</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>body, visibility, version</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PostView</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, created_at, updated_at, is_liked_by_me, is_edited</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ProfilePublic</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ProfileSelf</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RefreshRequest</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>refresh_token</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>RegisterRequest</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>email, password</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RegisterResponse</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>user, message</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
media upload + storage abstraction (local + S3-ready) + dedupe + attach-to-post
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -935,22 +935,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/media</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Unmute</t>
+          <t>Upload Media</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -958,32 +958,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Body_upload_media_api_v1_media_post</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mute</t>
+          <t>Delete Media</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1001,22 +1005,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>/api/v1/posts</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Create Post</t>
+          <t>Get Media</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1024,36 +1028,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>PostCreate</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>/api/v1/posts/by-author/{author_id}</t>
+          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>List By Author</t>
+          <t>Attach To Post</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1076,17 +1076,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Delete Post</t>
+          <t>Unmute</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1104,22 +1104,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Get Post</t>
+          <t>Mute</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1130,24 +1130,24 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/posts</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Update Post</t>
+          <t>Create Post</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1162,12 +1162,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>PostUpdate</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -1179,17 +1179,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/by-author/{author_id}</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>List Comments</t>
+          <t>List By Author</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1207,22 +1207,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Create Comment</t>
+          <t>Delete Post</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1230,36 +1230,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>CommentCreate</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Get Post</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1270,29 +1266,29 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Update Post</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1300,32 +1296,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>PostUpdate</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>List Comments</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1333,11 +1333,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>ProfileUpdate</t>
-        </is>
-      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1347,22 +1343,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>Create Comment</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1370,27 +1366,31 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>CommentCreate</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1403,31 +1403,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>ConsentGrantRequest</t>
-        </is>
-      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1443,24 +1439,24 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1473,7 +1469,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1488,17 +1488,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1509,29 +1509,29 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>Grant Consent</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1539,32 +1539,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/users/me/consent/{channel}</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Revoke Consent</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1575,7 +1579,7 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1587,17 +1591,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/users/{user_id}</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>Get Profile</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1620,28 +1624,28 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1653,28 +1657,28 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/api/v1/users/{user_id}/follow-status</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Status Endpoint</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1686,28 +1690,28 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/api/v1/users/{user_id}/followers</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Followers</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1719,26 +1723,158 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/api/v1/users/{user_id}/following</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>Following</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>/health</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Liveness probe</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>/health/db</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Database readiness probe</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -1755,7 +1891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1795,7 +1931,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CommentCreate</t>
+          <t>Body_upload_media_api_v1_media_post</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1805,14 +1941,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>body, parent_id</t>
+          <t>file</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CommentPage</t>
+          <t>CommentCreate</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1822,14 +1958,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>body, parent_id</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CommentUpdate</t>
+          <t>CommentPage</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1839,14 +1975,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>body, version</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CommentView</t>
+          <t>CommentUpdate</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1856,14 +1992,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at, is_liked_by_me, is_edited, replies</t>
+          <t>body, version</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ConsentGrantRequest</t>
+          <t>CommentView</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1873,14 +2009,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at, is_liked_by_me, is_edited, replies</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ConsentList</t>
+          <t>ConsentGrantRequest</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1890,14 +2026,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>consents</t>
+          <t>channel</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ConsentRecord</t>
+          <t>ConsentList</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1907,14 +2043,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>channel, granted, granted_at, revoked_at</t>
+          <t>consents</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DeleteMeResponse</t>
+          <t>ConsentRecord</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1924,14 +2060,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>message, hard_delete_after</t>
+          <t>channel, granted, granted_at, revoked_at</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FollowCounts</t>
+          <t>DeleteMeResponse</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1941,14 +2077,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>followers, following</t>
+          <t>message, hard_delete_after</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FollowListPage</t>
+          <t>FollowCounts</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1958,14 +2094,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>followers, following</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FollowStatus</t>
+          <t>FollowListPage</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1975,14 +2111,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FollowUserView</t>
+          <t>FollowStatus</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1992,14 +2128,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url, followed_at</t>
+          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HTTPValidationError</t>
+          <t>FollowUserView</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2009,14 +2145,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>user_id, display_name, avatar_url, followed_at</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LikeUser</t>
+          <t>HTTPValidationError</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2026,14 +2162,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url</t>
+          <t>detail</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LikeUserPage</t>
+          <t>LikeUser</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2043,14 +2179,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>user_id, display_name, avatar_url</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>LikeUserPage</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2060,14 +2196,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LoginResponse</t>
+          <t>LoginRequest</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2077,14 +2213,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PostCreate</t>
+          <t>LoginResponse</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2094,14 +2230,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>body, visibility</t>
+          <t>user, tokens</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PostPage</t>
+          <t>MediaView</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2111,14 +2247,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PostUpdate</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2128,14 +2264,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>body, visibility, version</t>
+          <t>body, visibility</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PostView</t>
+          <t>PostPage</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2145,14 +2281,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>id, author_id, body, visibility, like_count, comment_count, media_count, created_at, updated_at, is_liked_by_me, is_edited</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>PostUpdate</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2162,14 +2298,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>body, visibility, version</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>PostView</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2179,14 +2315,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, created_at, updated_at, is_liked_by_me, is_edited</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>ProfilePublic</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2196,14 +2332,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>ProfileSelf</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2213,14 +2349,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2230,14 +2366,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>RefreshRequest</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2247,14 +2383,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>refresh_token</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>RegisterRequest</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2264,22 +2400,56 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>RegisterResponse</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>user, message</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
home feed v1 with Redis ZSET cache + invalidation + metrics
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -770,22 +770,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/feed/home</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Unfollow a user (idempotent)</t>
+          <t>Home Feed</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>feed</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -796,14 +796,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Follow a user (idempotent)</t>
+          <t>Unfollow a user (idempotent)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -836,22 +836,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Unlike</t>
+          <t>Follow a user (idempotent)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -869,7 +869,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Like</t>
+          <t>Unlike</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -902,17 +902,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>List Likers</t>
+          <t>Like</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -928,29 +928,29 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/api/v1/media</t>
+          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Upload Media</t>
+          <t>List Likers</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -958,31 +958,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Body_upload_media_api_v1_media_post</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}</t>
+          <t>/api/v1/media</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Delete Media</t>
+          <t>Upload Media</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -995,17 +991,21 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Body_upload_media_api_v1_media_post</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Get Media</t>
+          <t>Delete Media</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1031,24 +1031,24 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Attach To Post</t>
+          <t>Get Media</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1071,22 +1071,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Unmute</t>
+          <t>Attach To Post</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1097,14 +1097,14 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mute</t>
+          <t>Unmute</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1142,17 +1142,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>/api/v1/posts</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Create Post</t>
+          <t>Mute</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1160,31 +1160,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>PostCreate</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>/api/v1/posts/by-author/{author_id}</t>
+          <t>/api/v1/posts</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>List By Author</t>
+          <t>Create Post</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1197,27 +1193,31 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>PostCreate</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/posts/by-author/{author_id}</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Delete Post</t>
+          <t>List By Author</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1233,14 +1233,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Get Post</t>
+          <t>Delete Post</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1266,14 +1266,14 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Update Post</t>
+          <t>Get Post</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1296,11 +1296,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>PostUpdate</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1310,22 +1306,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>List Comments</t>
+          <t>Update Post</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1333,7 +1329,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>PostUpdate</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1343,7 +1343,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Create Comment</t>
+          <t>List Comments</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1366,36 +1366,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>CommentCreate</t>
-        </is>
-      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Create Comment</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1403,17 +1399,21 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>CommentCreate</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1446,7 +1446,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1469,31 +1469,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>ProfileUpdate</t>
-        </is>
-      </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1506,17 +1502,21 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1539,31 +1539,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>ConsentGrantRequest</t>
-        </is>
-      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Grant Consent</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1576,27 +1572,31 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/users/me/consent/{channel}</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>Revoke Consent</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1612,7 +1612,7 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1624,17 +1624,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/users/{user_id}</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Get Profile</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1657,12 +1657,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1690,12 +1690,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/users/{user_id}/follow-status</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Status Endpoint</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1723,12 +1723,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/users/{user_id}/followers</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>Followers</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1756,28 +1756,28 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/{user_id}/following</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Following</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1789,12 +1789,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/health</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Liveness probe</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1822,12 +1822,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/health/db</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Database readiness probe</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/health/ready</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>Readiness probe (aggregate)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1875,6 +1875,39 @@
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -1891,7 +1924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2169,7 +2202,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LikeUser</t>
+          <t>HomeFeedPage</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2179,14 +2212,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LikeUserPage</t>
+          <t>LikeUser</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2196,14 +2229,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>user_id, display_name, avatar_url</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>LikeUserPage</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2213,14 +2246,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LoginResponse</t>
+          <t>LoginRequest</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2230,14 +2263,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MediaView</t>
+          <t>LoginResponse</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2247,14 +2280,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
+          <t>user, tokens</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PostCreate</t>
+          <t>MediaView</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2264,14 +2297,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>body, visibility</t>
+          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PostPage</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2281,14 +2314,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>body, visibility</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PostUpdate</t>
+          <t>PostPage</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2298,14 +2331,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>body, visibility, version</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PostView</t>
+          <t>PostUpdate</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2315,14 +2348,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>id, author_id, body, visibility, like_count, comment_count, media_count, created_at, updated_at, is_liked_by_me, is_edited</t>
+          <t>body, visibility, version</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>PostView</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2332,14 +2365,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, created_at, updated_at, is_liked_by_me, is_edited</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>ProfilePublic</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2349,14 +2382,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>ProfileSelf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2366,14 +2399,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2383,14 +2416,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>RefreshRequest</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2400,14 +2433,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>refresh_token</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>RegisterRequest</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2417,14 +2450,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>RegisterResponse</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2434,22 +2467,39 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>user, message</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
explore feed with HN-style trending score + Celery Beat refresh
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -775,12 +775,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>/api/v1/feed/home</t>
+          <t>/api/v1/feed/explore</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Home Feed</t>
+          <t>Explore Feed</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -803,22 +803,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/feed/home</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Unfollow a user (idempotent)</t>
+          <t>Home Feed</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>feed</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -829,14 +829,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Follow a user (idempotent)</t>
+          <t>Unfollow a user (idempotent)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -869,22 +869,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Unlike</t>
+          <t>Follow a user (idempotent)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -902,7 +902,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Like</t>
+          <t>Unlike</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -935,17 +935,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>List Likers</t>
+          <t>Like</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -961,29 +961,29 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/api/v1/media</t>
+          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Upload Media</t>
+          <t>List Likers</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -991,31 +991,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Body_upload_media_api_v1_media_post</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}</t>
+          <t>/api/v1/media</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Delete Media</t>
+          <t>Upload Media</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1028,17 +1024,21 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Body_upload_media_api_v1_media_post</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Get Media</t>
+          <t>Delete Media</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1064,24 +1064,24 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Attach To Post</t>
+          <t>Get Media</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1104,22 +1104,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Unmute</t>
+          <t>Attach To Post</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1130,14 +1130,14 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mute</t>
+          <t>Unmute</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1175,17 +1175,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>/api/v1/posts</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Create Post</t>
+          <t>Mute</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1193,31 +1193,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>PostCreate</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>/api/v1/posts/by-author/{author_id}</t>
+          <t>/api/v1/posts</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>List By Author</t>
+          <t>Create Post</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1230,27 +1226,31 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>PostCreate</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/posts/by-author/{author_id}</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Delete Post</t>
+          <t>List By Author</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1266,14 +1266,14 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Get Post</t>
+          <t>Delete Post</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1299,14 +1299,14 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Update Post</t>
+          <t>Get Post</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1329,11 +1329,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>PostUpdate</t>
-        </is>
-      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1343,22 +1339,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>List Comments</t>
+          <t>Update Post</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1366,7 +1362,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>PostUpdate</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1376,7 +1376,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Create Comment</t>
+          <t>List Comments</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1399,36 +1399,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>CommentCreate</t>
-        </is>
-      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Create Comment</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1436,17 +1432,21 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>CommentCreate</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1479,7 +1479,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1502,31 +1502,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>ProfileUpdate</t>
-        </is>
-      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1539,17 +1535,21 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1572,31 +1572,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>ConsentGrantRequest</t>
-        </is>
-      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Grant Consent</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1609,27 +1605,31 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/users/me/consent/{channel}</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>Revoke Consent</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1645,7 +1645,7 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1657,17 +1657,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/users/{user_id}</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Get Profile</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1690,12 +1690,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1723,12 +1723,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/users/{user_id}/follow-status</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Status Endpoint</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1756,12 +1756,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/users/{user_id}/followers</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>Followers</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1789,28 +1789,28 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/{user_id}/following</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Following</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1822,12 +1822,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/health</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Liveness probe</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/health/db</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Database readiness probe</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1888,12 +1888,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/health/ready</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>Readiness probe (aggregate)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1908,6 +1908,39 @@
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -1924,7 +1957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2117,7 +2150,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FollowCounts</t>
+          <t>ExploreFeedPage</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2127,14 +2160,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>followers, following</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FollowListPage</t>
+          <t>FollowCounts</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2144,14 +2177,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>followers, following</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FollowStatus</t>
+          <t>FollowListPage</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2161,14 +2194,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FollowUserView</t>
+          <t>FollowStatus</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2178,14 +2211,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url, followed_at</t>
+          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HTTPValidationError</t>
+          <t>FollowUserView</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2195,14 +2228,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>user_id, display_name, avatar_url, followed_at</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HomeFeedPage</t>
+          <t>HTTPValidationError</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2212,14 +2245,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>items, next_cursor, cache_hit</t>
+          <t>detail</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>LikeUser</t>
+          <t>HomeFeedPage</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2229,14 +2262,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LikeUserPage</t>
+          <t>LikeUser</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2246,14 +2279,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>user_id, display_name, avatar_url</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>LikeUserPage</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2263,14 +2296,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>LoginResponse</t>
+          <t>LoginRequest</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2280,14 +2313,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MediaView</t>
+          <t>LoginResponse</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2297,14 +2330,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
+          <t>user, tokens</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PostCreate</t>
+          <t>MediaView</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2314,14 +2347,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>body, visibility</t>
+          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PostPage</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2331,14 +2364,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>body, visibility</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PostUpdate</t>
+          <t>PostPage</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2348,14 +2381,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>body, visibility, version</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PostView</t>
+          <t>PostUpdate</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2365,14 +2398,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>id, author_id, body, visibility, like_count, comment_count, media_count, created_at, updated_at, is_liked_by_me, is_edited</t>
+          <t>body, visibility, version</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>PostView</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2382,14 +2415,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, created_at, updated_at, is_liked_by_me, is_edited</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>ProfilePublic</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2399,14 +2432,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>ProfileSelf</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2416,14 +2449,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2433,14 +2466,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>RefreshRequest</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2450,14 +2483,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>refresh_token</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>RegisterRequest</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2467,14 +2500,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>RegisterResponse</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2484,22 +2517,39 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>user, message</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
in-app notifications (idempotent, block-aware, cursor-paginated)
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1203,22 +1203,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>/api/v1/posts</t>
+          <t>/api/v1/notifications</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Create Post</t>
+          <t>List Notifications</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1226,36 +1226,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>PostCreate</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/api/v1/posts/by-author/{author_id}</t>
+          <t>/api/v1/notifications/read-all</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>List By Author</t>
+          <t>Mark All Read</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1266,29 +1262,29 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/notifications/unread-count</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Delete Post</t>
+          <t>Unread Count</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1299,29 +1295,29 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/notifications/{notif_id}</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Get Post</t>
+          <t>Delete Notification</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1332,29 +1328,29 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/notifications/{notif_id}/read</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Update Post</t>
+          <t>Mark Read</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1362,11 +1358,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>PostUpdate</t>
-        </is>
-      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1376,22 +1368,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>List Comments</t>
+          <t>Create Post</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1399,32 +1391,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>PostCreate</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/by-author/{author_id}</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Create Comment</t>
+          <t>List By Author</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1432,14 +1428,10 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>CommentCreate</t>
-        </is>
-      </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1451,17 +1443,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Delete Post</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1472,7 +1464,7 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1484,17 +1476,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Get Post</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1505,7 +1497,7 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1517,17 +1509,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>Update Post</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1537,7 +1529,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>PostUpdate</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1554,17 +1546,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>List Comments</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1575,7 +1567,7 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1587,17 +1579,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>Create Comment</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1607,7 +1599,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>ConsentGrantRequest</t>
+          <t>CommentCreate</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1624,12 +1616,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1645,7 +1637,7 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -1657,12 +1649,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1678,29 +1670,29 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1708,7 +1700,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1723,17 +1719,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1744,29 +1740,29 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Grant Consent</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1774,32 +1770,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/users/me/consent/{channel}</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>Revoke Consent</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1810,7 +1810,7 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1822,28 +1822,28 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/{user_id}</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Get Profile</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1855,28 +1855,28 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1888,28 +1888,28 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/api/v1/users/{user_id}/follow-status</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Status Endpoint</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1921,26 +1921,191 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/api/v1/users/{user_id}/followers</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>Followers</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/following</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Following</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>/health</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Liveness probe</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>/health/db</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Database readiness probe</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -1957,7 +2122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2337,7 +2502,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MediaView</t>
+          <t>MarkReadResponse</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2347,14 +2512,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
+          <t>updated</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PostCreate</t>
+          <t>MediaView</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2364,14 +2529,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>body, visibility</t>
+          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PostPage</t>
+          <t>NotificationPage</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2388,7 +2553,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PostUpdate</t>
+          <t>NotificationView</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2398,14 +2563,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>body, visibility, version</t>
+          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PostView</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2415,14 +2580,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>id, author_id, body, visibility, like_count, comment_count, media_count, created_at, updated_at, is_liked_by_me, is_edited</t>
+          <t>body, visibility</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>PostPage</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2432,14 +2597,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>PostUpdate</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2449,14 +2614,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>body, visibility, version</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>PostView</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2466,14 +2631,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>ProfilePublic</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2483,14 +2648,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>ProfileSelf</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2500,14 +2665,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2517,14 +2682,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>RefreshRequest</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2534,22 +2699,90 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>refresh_token</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>RegisterRequest</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>email, password</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>RegisterResponse</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>user, message</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>UnreadCount</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>unread</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
WebSocket foundation (manager, Redis pub/sub bridge, presence, heartbeat)
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1611,22 +1611,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/presence/{user_id}</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Get Presence</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>presence</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1637,14 +1637,14 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1677,7 +1677,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1700,31 +1700,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>ProfileUpdate</t>
-        </is>
-      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1737,17 +1733,21 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1770,31 +1770,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>ConsentGrantRequest</t>
-        </is>
-      </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Grant Consent</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1807,27 +1803,31 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/users/me/consent/{channel}</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>Revoke Consent</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1843,7 +1843,7 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1855,17 +1855,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/users/{user_id}</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Get Profile</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1888,12 +1888,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1921,12 +1921,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/users/{user_id}/follow-status</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Status Endpoint</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1954,12 +1954,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/users/{user_id}/followers</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>Followers</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1987,28 +1987,28 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/{user_id}/following</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Following</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2020,12 +2020,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/health</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Liveness probe</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2053,12 +2053,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/health/db</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Database readiness probe</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2086,12 +2086,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/health/ready</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>Readiness probe (aggregate)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2106,6 +2106,39 @@
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2122,7 +2155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2638,7 +2671,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>PresenceView</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2648,14 +2681,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>user_id, online, connections</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>ProfilePublic</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2665,14 +2698,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>ProfileSelf</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2682,14 +2715,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2699,14 +2732,14 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>RefreshRequest</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2716,14 +2749,14 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>refresh_token</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>RegisterRequest</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2733,14 +2766,14 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>UnreadCount</t>
+          <t>RegisterResponse</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2750,14 +2783,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>unread</t>
+          <t>user, message</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>UnreadCount</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2767,22 +2800,39 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>unread</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
chat 1-1 (rooms, messages, read receipts, typing via WS)
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -705,17 +705,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/api/v1/comments/{comment_id}</t>
+          <t>/api/v1/chat/messages/{message_id}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Delete Comment</t>
+          <t>Delete Message</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -733,22 +733,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>/api/v1/comments/{comment_id}</t>
+          <t>/api/v1/chat/rooms</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Update Comment</t>
+          <t>List My Rooms</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -756,36 +756,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>CommentUpdate</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>/api/v1/feed/explore</t>
+          <t>/api/v1/chat/rooms/direct</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Explore Feed</t>
+          <t>Create Direct Room</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>feed</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -793,7 +789,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>DirectRoomCreate</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -808,17 +808,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>/api/v1/feed/home</t>
+          <t>/api/v1/chat/rooms/{room_id}</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Home Feed</t>
+          <t>Get Room</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>feed</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -836,22 +836,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/messages</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Unfollow a user (idempotent)</t>
+          <t>List Messages</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -862,7 +862,7 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -874,17 +874,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/messages</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Follow a user (idempotent)</t>
+          <t>Send Message</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -892,32 +892,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>MessageCreate</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/read</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Unlike</t>
+          <t>Mark Read</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -925,32 +929,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ReadRequest</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/read-receipts</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Like</t>
+          <t>List Read Receipts</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -961,29 +969,29 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
+          <t>/api/v1/chat/rooms/{room_id}/typing</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>List Likers</t>
+          <t>Typing</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -994,29 +1002,29 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>/api/v1/media</t>
+          <t>/api/v1/chat/rooms/{room_id}/unread-count</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Upload Media</t>
+          <t>Unread Count</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1024,14 +1032,10 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Body_upload_media_api_v1_media_post</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1043,17 +1047,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}</t>
+          <t>/api/v1/comments/{comment_id}</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Delete Media</t>
+          <t>Delete Comment</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1071,22 +1075,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}</t>
+          <t>/api/v1/comments/{comment_id}</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Get Media</t>
+          <t>Update Comment</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1094,7 +1098,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>CommentUpdate</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1104,22 +1112,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
+          <t>/api/v1/feed/explore</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Attach To Post</t>
+          <t>Explore Feed</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>feed</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1137,22 +1145,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/feed/home</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Unmute</t>
+          <t>Home Feed</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>feed</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1163,24 +1171,24 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mute</t>
+          <t>Unfollow a user (idempotent)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1203,22 +1211,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>/api/v1/notifications</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>List Notifications</t>
+          <t>Follow a user (idempotent)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1229,29 +1237,29 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/read-all</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mark All Read</t>
+          <t>Unlike</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1262,29 +1270,29 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/unread-count</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Unread Count</t>
+          <t>Like</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1295,29 +1303,29 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}</t>
+          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Delete Notification</t>
+          <t>List Likers</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1328,7 +1336,7 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1340,17 +1348,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}/read</t>
+          <t>/api/v1/media</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mark Read</t>
+          <t>Upload Media</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1358,32 +1366,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Body_upload_media_api_v1_media_post</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>/api/v1/posts</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Create Post</t>
+          <t>Delete Media</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1391,14 +1403,10 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>PostCreate</t>
-        </is>
-      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1410,17 +1418,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>/api/v1/posts/by-author/{author_id}</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>List By Author</t>
+          <t>Get Media</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1438,22 +1446,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Delete Post</t>
+          <t>Attach To Post</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1464,29 +1472,29 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Get Post</t>
+          <t>Unmute</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1497,29 +1505,29 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Update Post</t>
+          <t>Mute</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1527,14 +1535,10 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>PostUpdate</t>
-        </is>
-      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1546,17 +1550,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/notifications</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>List Comments</t>
+          <t>List Notifications</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1579,17 +1583,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/notifications/read-all</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Create Comment</t>
+          <t>Mark All Read</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1597,14 +1601,10 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>CommentCreate</t>
-        </is>
-      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -1616,17 +1616,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>/api/v1/presence/{user_id}</t>
+          <t>/api/v1/notifications/unread-count</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Get Presence</t>
+          <t>Unread Count</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>presence</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1637,7 +1637,7 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -1649,17 +1649,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/notifications/{notif_id}</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Delete Notification</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1670,29 +1670,29 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/notifications/{notif_id}/read</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Mark Read</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1703,29 +1703,29 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>Create Post</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1735,12 +1735,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -1752,17 +1752,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/posts/by-author/{author_id}</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>List By Author</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1773,29 +1773,29 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>Delete Post</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1803,36 +1803,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>ConsentGrantRequest</t>
-        </is>
-      </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Get Post</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1843,29 +1839,29 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>Update Post</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1873,7 +1869,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>PostUpdate</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1888,17 +1888,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>List Comments</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1916,22 +1916,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>Create Comment</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1939,10 +1939,14 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>CommentCreate</t>
+        </is>
+      </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -1954,17 +1958,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/presence/{user_id}</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Get Presence</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>presence</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1982,22 +1986,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2008,7 +2012,7 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -2020,22 +2024,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -2048,33 +2052,37 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>public</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2086,22 +2094,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -2114,31 +2122,365 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>/api/v1/users/me/consent</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Grant Consent</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>201, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>/api/v1/users/me/consent/{channel}</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Revoke Consent</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>204, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Get Profile</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/follow-status</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Status Endpoint</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/followers</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Followers</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/following</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Following</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>/health</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Liveness probe</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>/health/db</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Database readiness probe</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
         <is>
           <t>/health/redis</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>Redis readiness probe</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>health</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>public</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr">
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2155,7 +2497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2348,7 +2690,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ExploreFeedPage</t>
+          <t>DirectRoomCreate</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2358,14 +2700,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>items, next_cursor, cache_hit</t>
+          <t>other_user_id</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FollowCounts</t>
+          <t>ExploreFeedPage</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2375,14 +2717,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>followers, following</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FollowListPage</t>
+          <t>FollowCounts</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2392,14 +2734,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>followers, following</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FollowStatus</t>
+          <t>FollowListPage</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2409,14 +2751,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FollowUserView</t>
+          <t>FollowStatus</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2426,14 +2768,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url, followed_at</t>
+          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HTTPValidationError</t>
+          <t>FollowUserView</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2443,14 +2785,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>user_id, display_name, avatar_url, followed_at</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HomeFeedPage</t>
+          <t>HTTPValidationError</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2460,14 +2802,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>items, next_cursor, cache_hit</t>
+          <t>detail</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LikeUser</t>
+          <t>HomeFeedPage</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2477,14 +2819,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LikeUserPage</t>
+          <t>LikeUser</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2494,14 +2836,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>user_id, display_name, avatar_url</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>LikeUserPage</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2511,14 +2853,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LoginResponse</t>
+          <t>LoginRequest</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2528,14 +2870,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MarkReadResponse</t>
+          <t>LoginResponse</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2545,14 +2887,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>updated</t>
+          <t>user, tokens</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MediaView</t>
+          <t>MarkReadResponse</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2562,14 +2904,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
+          <t>updated</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NotificationPage</t>
+          <t>MediaView</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2579,14 +2921,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NotificationView</t>
+          <t>MemberReadState</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2596,14 +2938,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
+          <t>user_id, last_read_message_id</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PostCreate</t>
+          <t>MessageCreate</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2613,14 +2955,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>body, visibility</t>
+          <t>body, media_id</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PostPage</t>
+          <t>MessagePage</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2637,7 +2979,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PostUpdate</t>
+          <t>MessageView</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2647,14 +2989,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>body, visibility, version</t>
+          <t>id, room_id, sender_id, body, media_id, created_at, is_edited</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PostView</t>
+          <t>NotificationPage</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2664,14 +3006,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PresenceView</t>
+          <t>NotificationView</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2681,14 +3023,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>user_id, online, connections</t>
+          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2698,14 +3040,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>body, visibility</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>PostPage</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2715,14 +3057,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>PostUpdate</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2732,14 +3074,14 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>body, visibility, version</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>PostView</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2749,14 +3091,14 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>PresenceView</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2766,14 +3108,14 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>user_id, online, connections</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>ProfilePublic</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2783,14 +3125,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>UnreadCount</t>
+          <t>ProfileSelf</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2800,14 +3142,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>unread</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2817,22 +3159,158 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>ReadReceiptsList</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>members</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ReadRequest</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>message_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>RefreshRequest</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>refresh_token</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>RegisterRequest</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>email, password</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>RegisterResponse</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>user, message</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>RoomView</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>id, type, title, created_at, updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>UnreadCount</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>unread</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
chat group rooms + media messages + WS room subscriptions
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -803,17 +803,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}</t>
+          <t>/api/v1/chat/rooms/group</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Get Room</t>
+          <t>Create Group</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -826,10 +826,14 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>GroupRoomCreate</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -841,12 +845,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/messages</t>
+          <t>/api/v1/chat/rooms/{room_id}</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>List Messages</t>
+          <t>Get Room</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -869,17 +873,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/messages</t>
+          <t>/api/v1/chat/rooms/{room_id}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Send Message</t>
+          <t>Update Room</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -894,29 +898,29 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>MessageCreate</t>
+          <t>RoomUpdate</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/read</t>
+          <t>/api/v1/chat/rooms/{room_id}/members</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mark Read</t>
+          <t>List Members</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -929,11 +933,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>ReadRequest</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -943,17 +943,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/read-receipts</t>
+          <t>/api/v1/chat/rooms/{room_id}/members</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>List Read Receipts</t>
+          <t>Add Member</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -966,27 +966,31 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>AddMemberRequest</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/typing</t>
+          <t>/api/v1/chat/rooms/{room_id}/members/{target_id}</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Typing</t>
+          <t>Remove Member</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1014,12 +1018,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/unread-count</t>
+          <t>/api/v1/chat/rooms/{room_id}/messages</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Unread Count</t>
+          <t>List Messages</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1042,22 +1046,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>/api/v1/comments/{comment_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/messages</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Delete Comment</t>
+          <t>Send Message</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1065,32 +1069,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>MessageCreate</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>/api/v1/comments/{comment_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/read</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Update Comment</t>
+          <t>Mark Read</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1100,7 +1108,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>CommentUpdate</t>
+          <t>ReadRequest</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1117,17 +1125,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>/api/v1/feed/explore</t>
+          <t>/api/v1/chat/rooms/{room_id}/read-receipts</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Explore Feed</t>
+          <t>List Read Receipts</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>feed</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1145,22 +1153,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>/api/v1/feed/home</t>
+          <t>/api/v1/chat/rooms/{room_id}/typing</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Home Feed</t>
+          <t>Typing</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>feed</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1171,29 +1179,29 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/unread-count</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Unfollow a user (idempotent)</t>
+          <t>Unread Count</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1204,29 +1212,29 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/comments/{comment_id}</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Follow a user (idempotent)</t>
+          <t>Delete Comment</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1244,22 +1252,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}</t>
+          <t>/api/v1/comments/{comment_id}</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Unlike</t>
+          <t>Update Comment</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1267,32 +1275,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>CommentUpdate</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}</t>
+          <t>/api/v1/feed/explore</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Like</t>
+          <t>Explore Feed</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>feed</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1303,7 +1315,7 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1315,17 +1327,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
+          <t>/api/v1/feed/home</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>List Likers</t>
+          <t>Home Feed</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>feed</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1343,22 +1355,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>/api/v1/media</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Upload Media</t>
+          <t>Unfollow a user (idempotent)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1366,36 +1378,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Body_upload_media_api_v1_media_post</t>
-        </is>
-      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Delete Media</t>
+          <t>Follow a user (idempotent)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1413,22 +1421,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Get Media</t>
+          <t>Unlike</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1439,7 +1447,7 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1451,17 +1459,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Attach To Post</t>
+          <t>Like</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1472,29 +1480,29 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Unmute</t>
+          <t>List Likers</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1505,7 +1513,7 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1517,17 +1525,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/media</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Mute</t>
+          <t>Upload Media</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1535,32 +1543,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Body_upload_media_api_v1_media_post</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>/api/v1/notifications</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>List Notifications</t>
+          <t>Delete Media</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1571,29 +1583,29 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/read-all</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Mark All Read</t>
+          <t>Get Media</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1604,29 +1616,29 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/unread-count</t>
+          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Unread Count</t>
+          <t>Attach To Post</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1637,7 +1649,7 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1649,17 +1661,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Delete Notification</t>
+          <t>Unmute</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1682,17 +1694,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}/read</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Mark Read</t>
+          <t>Mute</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1703,29 +1715,29 @@
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/api/v1/posts</t>
+          <t>/api/v1/notifications</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Create Post</t>
+          <t>List Notifications</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1733,36 +1745,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>PostCreate</t>
-        </is>
-      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>/api/v1/posts/by-author/{author_id}</t>
+          <t>/api/v1/notifications/read-all</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>List By Author</t>
+          <t>Mark All Read</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1773,29 +1781,29 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/notifications/unread-count</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Delete Post</t>
+          <t>Unread Count</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1806,29 +1814,29 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/notifications/{notif_id}</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Get Post</t>
+          <t>Delete Notification</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1839,29 +1847,29 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/notifications/{notif_id}/read</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Update Post</t>
+          <t>Mark Read</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1869,11 +1877,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>PostUpdate</t>
-        </is>
-      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1883,22 +1887,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>List Comments</t>
+          <t>Create Post</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1906,32 +1910,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>PostCreate</t>
+        </is>
+      </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/by-author/{author_id}</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Create Comment</t>
+          <t>List By Author</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1939,36 +1947,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>CommentCreate</t>
-        </is>
-      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>/api/v1/presence/{user_id}</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Get Presence</t>
+          <t>Delete Post</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>presence</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1979,29 +1983,29 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Get Post</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2012,29 +2016,29 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Update Post</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2042,32 +2046,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>PostUpdate</t>
+        </is>
+      </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>List Comments</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2075,11 +2083,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>ProfileUpdate</t>
-        </is>
-      </c>
+      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -2089,22 +2093,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>Create Comment</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2112,32 +2116,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>CommentCreate</t>
+        </is>
+      </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/presence/{user_id}</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>Get Presence</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>presence</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2145,14 +2153,10 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>ConsentGrantRequest</t>
-        </is>
-      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2164,12 +2168,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2185,7 +2189,7 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -2197,12 +2201,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2218,29 +2222,29 @@
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2248,7 +2252,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="G54" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -2263,17 +2271,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2284,29 +2292,29 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Grant Consent</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2314,32 +2322,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/users/me/consent/{channel}</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>Revoke Consent</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2350,7 +2362,7 @@
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -2362,28 +2374,28 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/{user_id}</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Get Profile</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2395,28 +2407,28 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2428,28 +2440,28 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/api/v1/users/{user_id}/follow-status</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Status Endpoint</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2461,26 +2473,191 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/api/v1/users/{user_id}/followers</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>Followers</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/following</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Following</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>/health</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Liveness probe</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>/health/db</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Database readiness probe</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2497,7 +2674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2520,7 +2697,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AuthTokens</t>
+          <t>AddMemberRequest</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2530,14 +2707,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>access_token, refresh_token, token_type, expires_in</t>
+          <t>user_id</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Body_upload_media_api_v1_media_post</t>
+          <t>AuthTokens</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2547,14 +2724,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>access_token, refresh_token, token_type, expires_in</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CommentCreate</t>
+          <t>Body_upload_media_api_v1_media_post</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2564,14 +2741,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>body, parent_id</t>
+          <t>file</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CommentPage</t>
+          <t>CommentCreate</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2581,14 +2758,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>body, parent_id</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CommentUpdate</t>
+          <t>CommentPage</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2598,14 +2775,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>body, version</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CommentView</t>
+          <t>CommentUpdate</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2615,14 +2792,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at, is_liked_by_me, is_edited, replies</t>
+          <t>body, version</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ConsentGrantRequest</t>
+          <t>CommentView</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2632,14 +2809,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at, is_liked_by_me, is_edited, replies</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ConsentList</t>
+          <t>ConsentGrantRequest</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2649,14 +2826,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>consents</t>
+          <t>channel</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ConsentRecord</t>
+          <t>ConsentList</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2666,14 +2843,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>channel, granted, granted_at, revoked_at</t>
+          <t>consents</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DeleteMeResponse</t>
+          <t>ConsentRecord</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2683,14 +2860,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>message, hard_delete_after</t>
+          <t>channel, granted, granted_at, revoked_at</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DirectRoomCreate</t>
+          <t>DeleteMeResponse</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2700,14 +2877,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>other_user_id</t>
+          <t>message, hard_delete_after</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ExploreFeedPage</t>
+          <t>DirectRoomCreate</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2717,14 +2894,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>items, next_cursor, cache_hit</t>
+          <t>other_user_id</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FollowCounts</t>
+          <t>ExploreFeedPage</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2734,14 +2911,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>followers, following</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FollowListPage</t>
+          <t>FollowCounts</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2751,14 +2928,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>followers, following</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FollowStatus</t>
+          <t>FollowListPage</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2768,14 +2945,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FollowUserView</t>
+          <t>FollowStatus</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2785,14 +2962,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url, followed_at</t>
+          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HTTPValidationError</t>
+          <t>FollowUserView</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2802,14 +2979,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>user_id, display_name, avatar_url, followed_at</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HomeFeedPage</t>
+          <t>GroupRoomCreate</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2819,14 +2996,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>items, next_cursor, cache_hit</t>
+          <t>title, member_ids</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LikeUser</t>
+          <t>HTTPValidationError</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2836,14 +3013,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url</t>
+          <t>detail</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>LikeUserPage</t>
+          <t>HomeFeedPage</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2853,14 +3030,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>LikeUser</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2870,14 +3047,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>user_id, display_name, avatar_url</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LoginResponse</t>
+          <t>LikeUserPage</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2887,14 +3064,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MarkReadResponse</t>
+          <t>LoginRequest</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2904,14 +3081,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>updated</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MediaView</t>
+          <t>LoginResponse</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2921,14 +3098,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
+          <t>user, tokens</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MemberReadState</t>
+          <t>MarkReadResponse</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2938,14 +3115,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>user_id, last_read_message_id</t>
+          <t>updated</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MessageCreate</t>
+          <t>MediaView</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2955,14 +3132,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>body, media_id</t>
+          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MessagePage</t>
+          <t>MemberReadState</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2972,14 +3149,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>user_id, last_read_message_id</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MessageView</t>
+          <t>MessageCreate</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2989,14 +3166,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>id, room_id, sender_id, body, media_id, created_at, is_edited</t>
+          <t>body, media_id</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>NotificationPage</t>
+          <t>MessagePage</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3013,7 +3190,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NotificationView</t>
+          <t>MessageView</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3023,14 +3200,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
+          <t>id, room_id, sender_id, body, media_id, created_at, is_edited</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PostCreate</t>
+          <t>NotificationPage</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3040,14 +3217,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>body, visibility</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PostPage</t>
+          <t>NotificationView</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3057,14 +3234,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PostUpdate</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3074,14 +3251,14 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>body, visibility, version</t>
+          <t>body, visibility</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PostView</t>
+          <t>PostPage</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3091,14 +3268,14 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PresenceView</t>
+          <t>PostUpdate</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3108,14 +3285,14 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>user_id, online, connections</t>
+          <t>body, visibility, version</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>PostView</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3125,14 +3302,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>PresenceView</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3142,14 +3319,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>user_id, online, connections</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>ProfilePublic</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3159,14 +3336,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ReadReceiptsList</t>
+          <t>ProfileSelf</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3176,14 +3353,14 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>members</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ReadRequest</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3193,14 +3370,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>message_id</t>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>ReadReceiptsList</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3210,14 +3387,14 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>members</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>ReadRequest</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3227,14 +3404,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>message_id</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>RefreshRequest</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3244,14 +3421,14 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>refresh_token</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>RoomView</t>
+          <t>RegisterRequest</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3261,14 +3438,14 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>id, type, title, created_at, updated_at</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>UnreadCount</t>
+          <t>RegisterResponse</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3278,14 +3455,14 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>unread</t>
+          <t>user, message</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>RoomMemberView</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3295,22 +3472,107 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>user_id, role, joined_at</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>RoomMembersList</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>members</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>RoomUpdate</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>title, version</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>RoomView</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>id, type, title, created_at, updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>UnreadCount</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>unread</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
moderation (reports queue, status lifecycle, WS resolve)
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1656,22 +1656,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/moderation/reports</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Unmute</t>
+          <t>List Reports</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>moderation</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1682,7 +1682,7 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1694,17 +1694,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/moderation/reports</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Mute</t>
+          <t>Create Report</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>moderation</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1712,32 +1712,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>ReportCreate</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/api/v1/notifications</t>
+          <t>/api/v1/moderation/reports/{report_id}</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>List Notifications</t>
+          <t>Update Report</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>moderation</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1745,7 +1749,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>ReportUpdate</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1755,22 +1763,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/read-all</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Mark All Read</t>
+          <t>Unmute</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1781,29 +1789,29 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/unread-count</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Unread Count</t>
+          <t>Mute</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1814,24 +1822,24 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}</t>
+          <t>/api/v1/notifications</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Delete Notification</t>
+          <t>List Notifications</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1847,7 +1855,7 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1867,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}/read</t>
+          <t>/api/v1/notifications/read-all</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mark Read</t>
+          <t>Mark All Read</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1880,29 +1888,29 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/api/v1/posts</t>
+          <t>/api/v1/notifications/unread-count</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Create Post</t>
+          <t>Unread Count</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1910,36 +1918,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>PostCreate</t>
-        </is>
-      </c>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>/api/v1/posts/by-author/{author_id}</t>
+          <t>/api/v1/notifications/{notif_id}</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>List By Author</t>
+          <t>Delete Notification</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1950,29 +1954,29 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/notifications/{notif_id}/read</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Delete Post</t>
+          <t>Mark Read</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1983,24 +1987,24 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/posts</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Get Post</t>
+          <t>Create Post</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2013,27 +2017,31 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>PostCreate</t>
+        </is>
+      </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/posts/by-author/{author_id}</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Update Post</t>
+          <t>List By Author</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2046,11 +2054,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>PostUpdate</t>
-        </is>
-      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -2060,22 +2064,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>List Comments</t>
+          <t>Delete Post</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2086,29 +2090,29 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Create Comment</t>
+          <t>Get Post</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2116,36 +2120,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>CommentCreate</t>
-        </is>
-      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>/api/v1/presence/{user_id}</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Get Presence</t>
+          <t>Update Post</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>presence</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2153,7 +2153,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>PostUpdate</t>
+        </is>
+      </c>
       <c r="G51" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -2163,22 +2167,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>List Comments</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2189,29 +2193,29 @@
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Create Comment</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2219,32 +2223,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>CommentCreate</t>
+        </is>
+      </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/presence/{user_id}</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>Get Presence</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>presence</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2252,11 +2260,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>ProfileUpdate</t>
-        </is>
-      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -2266,17 +2270,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2299,17 +2303,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2322,31 +2326,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>ConsentGrantRequest</t>
-        </is>
-      </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2359,10 +2359,14 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2374,12 +2378,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2395,29 +2399,29 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Grant Consent</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2425,32 +2429,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/users/me/consent/{channel}</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>Revoke Consent</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2461,7 +2469,7 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -2473,17 +2481,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/users/{user_id}</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Get Profile</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2506,12 +2514,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2539,28 +2547,28 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/{user_id}/follow-status</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Status Endpoint</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2572,28 +2580,28 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/api/v1/users/{user_id}/followers</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Followers</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2605,28 +2613,28 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/api/v1/users/{user_id}/following</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Following</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2638,12 +2646,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/health</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>Liveness probe</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2658,6 +2666,105 @@
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>/health/db</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Database readiness probe</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2674,7 +2781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3462,7 +3569,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>RoomMemberView</t>
+          <t>ReportCreate</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3472,14 +3579,14 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>user_id, role, joined_at</t>
+          <t>target_type, target_id, reason, details</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>RoomMembersList</t>
+          <t>ReportPage</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3489,31 +3596,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>members</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>RoomUpdate</t>
+          <t>ReportStatus</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>title, version</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>RoomView</t>
+          <t>ReportUpdate</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3523,14 +3626,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>id, type, title, created_at, updated_at</t>
+          <t>status, resolution_note, version</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>UnreadCount</t>
+          <t>ReportView</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3540,14 +3643,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>unread</t>
+          <t>id, reporter_id, target_type, target_id, reason, details, status, reviewer_id, resolution_note, resolved_at, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>RoomMemberView</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3557,22 +3660,107 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>user_id, role, joined_at</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>RoomMembersList</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>members</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>RoomUpdate</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>title, version</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>RoomView</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>id, type, title, created_at, updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>UnreadCount</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>unread</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
GDPR (export, schedule/cancel delete, retention jobs)
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,34 +457,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>/api/v1/auth/login</t>
+          <t>/api/v1/audit</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>List All Audit</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>auth</t>
+          <t>audit</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>public</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>LoginRequest</t>
-        </is>
-      </c>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -494,22 +490,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>/api/v1/auth/logout</t>
+          <t>/api/v1/audit/me</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Logout</t>
+          <t>My Audit</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>auth</t>
+          <t>audit</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -520,24 +516,24 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>/api/v1/auth/me</t>
+          <t>/api/v1/auth/login</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Me</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -547,13 +543,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>LoginRequest</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -565,12 +565,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>/api/v1/auth/refresh</t>
+          <t>/api/v1/auth/logout</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Refresh</t>
+          <t>Logout</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -580,34 +580,30 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>public</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>RefreshRequest</t>
-        </is>
-      </c>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>/api/v1/auth/register</t>
+          <t>/api/v1/auth/me</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Register</t>
+          <t>Me</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -617,50 +613,50 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>public</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>RegisterRequest</t>
-        </is>
-      </c>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>/api/v1/blocks/{user_id}</t>
+          <t>/api/v1/auth/refresh</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Unblock</t>
+          <t>Refresh</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>auth</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>RefreshRequest</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -672,28 +668,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>/api/v1/blocks/{user_id}</t>
+          <t>/api/v1/auth/register</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Block</t>
+          <t>Register</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>auth</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>RegisterRequest</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -705,17 +705,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/api/v1/chat/messages/{message_id}</t>
+          <t>/api/v1/blocks/{user_id}</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Delete Message</t>
+          <t>Unblock</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>chat</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -733,22 +733,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms</t>
+          <t>/api/v1/blocks/{user_id}</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>List My Rooms</t>
+          <t>Block</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>chat</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -759,24 +759,24 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/direct</t>
+          <t>/api/v1/chat/messages/{message_id}</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Create Direct Room</t>
+          <t>Delete Message</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -789,31 +789,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>DirectRoomCreate</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/group</t>
+          <t>/api/v1/chat/rooms</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Create Group</t>
+          <t>List My Rooms</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -826,31 +822,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>GroupRoomCreate</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}</t>
+          <t>/api/v1/chat/rooms/direct</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Get Room</t>
+          <t>Create Direct Room</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -863,7 +855,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>DirectRoomCreate</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -873,17 +869,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}</t>
+          <t>/api/v1/chat/rooms/group</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Update Room</t>
+          <t>Create Group</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -898,12 +894,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>RoomUpdate</t>
+          <t>GroupRoomCreate</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -915,12 +911,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/members</t>
+          <t>/api/v1/chat/rooms/{room_id}</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>List Members</t>
+          <t>Get Room</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -943,17 +939,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/members</t>
+          <t>/api/v1/chat/rooms/{room_id}</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Add Member</t>
+          <t>Update Room</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -968,29 +964,29 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>AddMemberRequest</t>
+          <t>RoomUpdate</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/members/{target_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/members</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Remove Member</t>
+          <t>List Members</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1006,24 +1002,24 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/messages</t>
+          <t>/api/v1/chat/rooms/{room_id}/members</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>List Messages</t>
+          <t>Add Member</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1036,27 +1032,31 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>AddMemberRequest</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/messages</t>
+          <t>/api/v1/chat/rooms/{room_id}/members/{target_id}</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Send Message</t>
+          <t>Remove Member</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1069,31 +1069,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>MessageCreate</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/read</t>
+          <t>/api/v1/chat/rooms/{room_id}/messages</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mark Read</t>
+          <t>List Messages</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1106,11 +1102,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>ReadRequest</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1120,17 +1112,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/read-receipts</t>
+          <t>/api/v1/chat/rooms/{room_id}/messages</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>List Read Receipts</t>
+          <t>Send Message</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1143,10 +1135,14 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>MessageCreate</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -1158,12 +1154,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/typing</t>
+          <t>/api/v1/chat/rooms/{room_id}/read</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Typing</t>
+          <t>Mark Read</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1176,10 +1172,14 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>ReadRequest</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1191,12 +1191,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/unread-count</t>
+          <t>/api/v1/chat/rooms/{room_id}/read-receipts</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Unread Count</t>
+          <t>List Read Receipts</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1219,22 +1219,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>/api/v1/comments/{comment_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/typing</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Delete Comment</t>
+          <t>Typing</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1252,22 +1252,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/api/v1/comments/{comment_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/unread-count</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Update Comment</t>
+          <t>Unread Count</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1275,11 +1275,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>CommentUpdate</t>
-        </is>
-      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1289,22 +1285,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>/api/v1/feed/explore</t>
+          <t>/api/v1/comments/{comment_id}</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Explore Feed</t>
+          <t>Delete Comment</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>feed</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1315,29 +1311,29 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>/api/v1/feed/home</t>
+          <t>/api/v1/comments/{comment_id}</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Home Feed</t>
+          <t>Update Comment</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>feed</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1345,7 +1341,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>CommentUpdate</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1355,22 +1355,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/feed/explore</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Unfollow a user (idempotent)</t>
+          <t>Explore Feed</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>feed</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1381,29 +1381,29 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/feed/home</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Follow a user (idempotent)</t>
+          <t>Home Feed</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>feed</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1414,7 +1414,7 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1426,17 +1426,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Unlike</t>
+          <t>Unfollow a user (idempotent)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1459,17 +1459,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Like</t>
+          <t>Follow a user (idempotent)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1487,22 +1487,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
+          <t>/api/v1/gdpr/cancel-delete</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>List Likers</t>
+          <t>Cancel Deletion</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>gdpr</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1513,29 +1513,29 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>/api/v1/media</t>
+          <t>/api/v1/gdpr/deletion-status</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Upload Media</t>
+          <t>Deletion Status</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>gdpr</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1543,36 +1543,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Body_upload_media_api_v1_media_post</t>
-        </is>
-      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}</t>
+          <t>/api/v1/gdpr/export</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Delete Media</t>
+          <t>Export Data</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>gdpr</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1583,29 +1579,29 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Get Media</t>
+          <t>Unlike</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1616,7 +1612,7 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1628,17 +1624,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Attach To Post</t>
+          <t>Like</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1649,7 +1645,7 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1661,17 +1657,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/api/v1/moderation/reports</t>
+          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>List Reports</t>
+          <t>List Likers</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>moderation</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1694,17 +1690,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/api/v1/moderation/reports</t>
+          <t>/api/v1/media</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Create Report</t>
+          <t>Upload Media</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>moderation</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1714,7 +1710,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>ReportCreate</t>
+          <t>Body_upload_media_api_v1_media_post</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1726,22 +1722,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/api/v1/moderation/reports/{report_id}</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Update Report</t>
+          <t>Delete Media</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>moderation</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1749,36 +1745,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>ReportUpdate</t>
-        </is>
-      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Unmute</t>
+          <t>Get Media</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1789,7 +1781,7 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1801,17 +1793,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mute</t>
+          <t>Attach To Post</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1822,7 +1814,7 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1834,17 +1826,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/api/v1/notifications</t>
+          <t>/api/v1/moderation/reports</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>List Notifications</t>
+          <t>List Reports</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>moderation</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1867,17 +1859,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/read-all</t>
+          <t>/api/v1/moderation/reports</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Mark All Read</t>
+          <t>Create Report</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>moderation</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1885,32 +1877,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>ReportCreate</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/unread-count</t>
+          <t>/api/v1/moderation/reports/{report_id}</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Unread Count</t>
+          <t>Update Report</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>moderation</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1918,10 +1914,14 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>ReportUpdate</t>
+        </is>
+      </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1933,17 +1933,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Delete Notification</t>
+          <t>Unmute</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1966,17 +1966,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}/read</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mark Read</t>
+          <t>Mute</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1987,29 +1987,29 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>/api/v1/posts</t>
+          <t>/api/v1/notifications</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Create Post</t>
+          <t>List Notifications</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2017,36 +2017,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>PostCreate</t>
-        </is>
-      </c>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>/api/v1/posts/by-author/{author_id}</t>
+          <t>/api/v1/notifications/read-all</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>List By Author</t>
+          <t>Mark All Read</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2057,29 +2053,29 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/notifications/unread-count</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Delete Post</t>
+          <t>Unread Count</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2090,29 +2086,29 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/notifications/{notif_id}</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Get Post</t>
+          <t>Delete Notification</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2123,29 +2119,29 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/notifications/{notif_id}/read</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Update Post</t>
+          <t>Mark Read</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2153,11 +2149,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>PostUpdate</t>
-        </is>
-      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -2167,22 +2159,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>List Comments</t>
+          <t>Create Post</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2190,32 +2182,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>PostCreate</t>
+        </is>
+      </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/by-author/{author_id}</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Create Comment</t>
+          <t>List By Author</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2223,36 +2219,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>CommentCreate</t>
-        </is>
-      </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>/api/v1/presence/{user_id}</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Get Presence</t>
+          <t>Delete Post</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>presence</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2263,29 +2255,29 @@
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Get Post</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2296,29 +2288,29 @@
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Update Post</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2326,32 +2318,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>PostUpdate</t>
+        </is>
+      </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>List Comments</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2359,11 +2355,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>ProfileUpdate</t>
-        </is>
-      </c>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -2373,22 +2365,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>Create Comment</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2396,32 +2388,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>CommentCreate</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/presence/{user_id}</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>Get Presence</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>presence</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2429,14 +2425,10 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>ConsentGrantRequest</t>
-        </is>
-      </c>
+      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2448,12 +2440,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2469,7 +2461,7 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -2481,12 +2473,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2502,29 +2494,29 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -2532,7 +2524,11 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="G62" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -2547,17 +2543,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2568,29 +2564,29 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Grant Consent</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2598,32 +2594,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/users/me/consent/{channel}</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>Revoke Consent</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2634,7 +2634,7 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -2646,28 +2646,28 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/{user_id}</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Get Profile</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2679,28 +2679,28 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2712,28 +2712,28 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/api/v1/users/{user_id}/follow-status</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Status Endpoint</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2745,26 +2745,191 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/api/v1/users/{user_id}/followers</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>Followers</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>/api/v1/users/{user_id}/following</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Following</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>follows</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>HTTPBearer</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>200, 422</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>/health</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Liveness probe</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>/health/db</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Database readiness probe</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2781,7 +2946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2821,7 +2986,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AuthTokens</t>
+          <t>AuditLogView</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2831,14 +2996,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>access_token, refresh_token, token_type, expires_in</t>
+          <t>id, actor_id, action, entity, entity_id, before, after, ip, user_agent, request_id, created_at</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Body_upload_media_api_v1_media_post</t>
+          <t>AuditPage</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2848,14 +3013,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CommentCreate</t>
+          <t>AuthTokens</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2865,14 +3030,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>body, parent_id</t>
+          <t>access_token, refresh_token, token_type, expires_in</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CommentPage</t>
+          <t>Body_upload_media_api_v1_media_post</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2882,14 +3047,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>file</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CommentUpdate</t>
+          <t>CancelResponse</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2899,14 +3064,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>body, version</t>
+          <t>message</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CommentView</t>
+          <t>CommentCreate</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2916,14 +3081,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at, is_liked_by_me, is_edited, replies</t>
+          <t>body, parent_id</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ConsentGrantRequest</t>
+          <t>CommentPage</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2933,14 +3098,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ConsentList</t>
+          <t>CommentUpdate</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2950,14 +3115,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>consents</t>
+          <t>body, version</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ConsentRecord</t>
+          <t>CommentView</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2967,14 +3132,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>channel, granted, granted_at, revoked_at</t>
+          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at, is_liked_by_me, is_edited, replies</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DeleteMeResponse</t>
+          <t>ConsentGrantRequest</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2984,14 +3149,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>message, hard_delete_after</t>
+          <t>channel</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DirectRoomCreate</t>
+          <t>ConsentList</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3001,14 +3166,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>other_user_id</t>
+          <t>consents</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ExploreFeedPage</t>
+          <t>ConsentRecord</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3018,14 +3183,14 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>items, next_cursor, cache_hit</t>
+          <t>channel, granted, granted_at, revoked_at</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FollowCounts</t>
+          <t>DeleteMeResponse</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3035,14 +3200,14 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>followers, following</t>
+          <t>message, hard_delete_after</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FollowListPage</t>
+          <t>DeletionStatusView</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3052,14 +3217,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>scheduled, scheduled_hard_delete_at, status</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FollowStatus</t>
+          <t>DirectRoomCreate</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3069,14 +3234,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
+          <t>other_user_id</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FollowUserView</t>
+          <t>ExploreFeedPage</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3086,14 +3251,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url, followed_at</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GroupRoomCreate</t>
+          <t>FollowCounts</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3103,14 +3268,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>title, member_ids</t>
+          <t>followers, following</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HTTPValidationError</t>
+          <t>FollowListPage</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3120,14 +3285,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HomeFeedPage</t>
+          <t>FollowStatus</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3137,14 +3302,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>items, next_cursor, cache_hit</t>
+          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LikeUser</t>
+          <t>FollowUserView</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3154,14 +3319,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url</t>
+          <t>user_id, display_name, avatar_url, followed_at</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LikeUserPage</t>
+          <t>GroupRoomCreate</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3171,14 +3336,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>title, member_ids</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>HTTPValidationError</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3188,14 +3353,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>detail</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>LoginResponse</t>
+          <t>HomeFeedPage</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3205,14 +3370,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MarkReadResponse</t>
+          <t>LikeUser</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3222,14 +3387,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>updated</t>
+          <t>user_id, display_name, avatar_url</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MediaView</t>
+          <t>LikeUserPage</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3239,14 +3404,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MemberReadState</t>
+          <t>LoginRequest</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3256,14 +3421,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>user_id, last_read_message_id</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MessageCreate</t>
+          <t>LoginResponse</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3273,14 +3438,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>body, media_id</t>
+          <t>user, tokens</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MessagePage</t>
+          <t>MarkReadResponse</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3290,14 +3455,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>updated</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MessageView</t>
+          <t>MediaView</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3307,14 +3472,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>id, room_id, sender_id, body, media_id, created_at, is_edited</t>
+          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>NotificationPage</t>
+          <t>MemberReadState</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3324,14 +3489,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>user_id, last_read_message_id</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>NotificationView</t>
+          <t>MessageCreate</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3341,14 +3506,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
+          <t>body, media_id</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PostCreate</t>
+          <t>MessagePage</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3358,14 +3523,14 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>body, visibility</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PostPage</t>
+          <t>MessageView</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3375,14 +3540,14 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>id, room_id, sender_id, body, media_id, created_at, is_edited</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PostUpdate</t>
+          <t>NotificationPage</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3392,14 +3557,14 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>body, visibility, version</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PostView</t>
+          <t>NotificationView</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3409,14 +3574,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited</t>
+          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PresenceView</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3426,14 +3591,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>user_id, online, connections</t>
+          <t>body, visibility</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>PostPage</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3443,14 +3608,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>PostUpdate</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3460,14 +3625,14 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>body, visibility, version</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>PostView</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3477,14 +3642,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ReadReceiptsList</t>
+          <t>PresenceView</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3494,14 +3659,14 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>members</t>
+          <t>user_id, online, connections</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ReadRequest</t>
+          <t>ProfilePublic</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3511,14 +3676,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>message_id</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>ProfileSelf</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3528,14 +3693,14 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3545,14 +3710,14 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>ReadReceiptsList</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3562,14 +3727,14 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>members</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ReportCreate</t>
+          <t>ReadRequest</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3579,14 +3744,14 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>target_type, target_id, reason, details</t>
+          <t>message_id</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ReportPage</t>
+          <t>RefreshRequest</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3596,27 +3761,31 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>refresh_token</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ReportStatus</t>
+          <t>RegisterRequest</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>email, password</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ReportUpdate</t>
+          <t>RegisterResponse</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3626,14 +3795,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>status, resolution_note, version</t>
+          <t>user, message</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ReportView</t>
+          <t>ReportCreate</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3643,14 +3812,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>id, reporter_id, target_type, target_id, reason, details, status, reviewer_id, resolution_note, resolved_at, created_at, updated_at</t>
+          <t>target_type, target_id, reason, details</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>RoomMemberView</t>
+          <t>ReportPage</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3660,31 +3829,27 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>user_id, role, joined_at</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>RoomMembersList</t>
+          <t>ReportStatus</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>members</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>RoomUpdate</t>
+          <t>ReportUpdate</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3694,14 +3859,14 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>title, version</t>
+          <t>status, resolution_note, version</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>RoomView</t>
+          <t>ReportView</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3711,14 +3876,14 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>id, type, title, created_at, updated_at</t>
+          <t>id, reporter_id, target_type, target_id, reason, details, status, reviewer_id, resolution_note, resolved_at, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>UnreadCount</t>
+          <t>RoomMemberView</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3728,14 +3893,14 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>unread</t>
+          <t>user_id, role, joined_at</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>RoomMembersList</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3745,22 +3910,90 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>members</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>RoomUpdate</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>title, version</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>RoomView</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>id, type, title, created_at, updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>UnreadCount</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>unread</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
circuit breakers (redis/smtp/s3) + graceful fallback + uniform rate-limit headers
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/health/circuit-breakers</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Circuit-breaker snapshot (admin-only)</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -2877,12 +2877,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/health/db</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Database readiness probe</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2910,12 +2910,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/health/ready</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>Readiness probe (aggregate)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2930,6 +2930,39 @@
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
         <is>
           <t>200</t>
         </is>

</xml_diff>

<commit_message>
idempotency keys + feature flag overrides (Redis) + admin flag API
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1421,22 +1421,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/flags</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Unfollow a user (idempotent)</t>
+          <t>List Flags</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>flags</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1447,7 +1447,7 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -1459,17 +1459,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/flags/{flag_name}/override</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Follow a user (idempotent)</t>
+          <t>Override Flag</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>flags</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1477,32 +1477,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>FlagOverride</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>/api/v1/gdpr/cancel-delete</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Cancel Deletion</t>
+          <t>Unfollow a user (idempotent)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>gdpr</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1513,29 +1517,29 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>/api/v1/gdpr/deletion-status</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Deletion Status</t>
+          <t>Follow a user (idempotent)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>gdpr</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1546,24 +1550,24 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>/api/v1/gdpr/export</t>
+          <t>/api/v1/gdpr/cancel-delete</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Export Data</t>
+          <t>Cancel Deletion</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1586,22 +1590,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}</t>
+          <t>/api/v1/gdpr/deletion-status</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Unlike</t>
+          <t>Deletion Status</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>gdpr</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1612,29 +1616,29 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}</t>
+          <t>/api/v1/gdpr/export</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Like</t>
+          <t>Export Data</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>gdpr</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1645,24 +1649,24 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>List Likers</t>
+          <t>Unlike</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1678,7 +1682,7 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1690,17 +1694,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/api/v1/media</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Upload Media</t>
+          <t>Like</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1708,36 +1712,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Body_upload_media_api_v1_media_post</t>
-        </is>
-      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}</t>
+          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Delete Media</t>
+          <t>List Likers</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1748,24 +1748,24 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}</t>
+          <t>/api/v1/media</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Get Media</t>
+          <t>Upload Media</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1778,27 +1778,31 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Body_upload_media_api_v1_media_post</t>
+        </is>
+      </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Attach To Post</t>
+          <t>Delete Media</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1814,7 +1818,7 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -1826,17 +1830,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/api/v1/moderation/reports</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>List Reports</t>
+          <t>Get Media</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>moderation</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1859,17 +1863,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/api/v1/moderation/reports</t>
+          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Create Report</t>
+          <t>Attach To Post</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>moderation</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1877,31 +1881,27 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>ReportCreate</t>
-        </is>
-      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/api/v1/moderation/reports/{report_id}</t>
+          <t>/api/v1/moderation/reports</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Update Report</t>
+          <t>List Reports</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1914,11 +1914,7 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>ReportUpdate</t>
-        </is>
-      </c>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1928,22 +1924,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/moderation/reports</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Unmute</t>
+          <t>Create Report</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>moderation</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1951,32 +1947,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>ReportCreate</t>
+        </is>
+      </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/moderation/reports/{report_id}</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mute</t>
+          <t>Update Report</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>moderation</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1984,32 +1984,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>ReportUpdate</t>
+        </is>
+      </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>/api/v1/notifications</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>List Notifications</t>
+          <t>Unmute</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2020,7 +2024,7 @@
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -2032,17 +2036,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/read-all</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Mark All Read</t>
+          <t>Mute</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2053,7 +2057,7 @@
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -2065,12 +2069,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/unread-count</t>
+          <t>/api/v1/notifications</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Unread Count</t>
+          <t>List Notifications</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2086,24 +2090,24 @@
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}</t>
+          <t>/api/v1/notifications/read-all</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Delete Notification</t>
+          <t>Mark All Read</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2119,24 +2123,24 @@
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}/read</t>
+          <t>/api/v1/notifications/unread-count</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Mark Read</t>
+          <t>Unread Count</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2152,29 +2156,29 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>/api/v1/posts</t>
+          <t>/api/v1/notifications/{notif_id}</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Create Post</t>
+          <t>Delete Notification</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2182,36 +2186,32 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>PostCreate</t>
-        </is>
-      </c>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>/api/v1/posts/by-author/{author_id}</t>
+          <t>/api/v1/notifications/{notif_id}/read</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>List By Author</t>
+          <t>Mark Read</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2229,17 +2229,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/posts</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Delete Post</t>
+          <t>Create Post</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2252,10 +2252,14 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>PostCreate</t>
+        </is>
+      </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -2267,12 +2271,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/posts/by-author/{author_id}</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Get Post</t>
+          <t>List By Author</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2295,7 +2299,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2305,7 +2309,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Update Post</t>
+          <t>Delete Post</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2318,14 +2322,10 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>PostUpdate</t>
-        </is>
-      </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -2337,17 +2337,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>List Comments</t>
+          <t>Get Post</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2365,22 +2365,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Create Comment</t>
+          <t>Update Post</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2390,12 +2390,12 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>CommentCreate</t>
+          <t>PostUpdate</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2407,17 +2407,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>/api/v1/presence/{user_id}</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Get Presence</t>
+          <t>List Comments</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>presence</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2435,22 +2435,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Create Comment</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2458,10 +2458,14 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>CommentCreate</t>
+        </is>
+      </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -2473,17 +2477,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/presence/{user_id}</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Get Presence</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>presence</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2494,14 +2498,14 @@
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2511,7 +2515,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2524,14 +2528,10 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>ProfileUpdate</t>
-        </is>
-      </c>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -2543,12 +2543,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2571,17 +2571,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2596,29 +2596,29 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>ConsentGrantRequest</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2634,24 +2634,24 @@
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>Grant Consent</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2664,32 +2664,36 @@
           <t>HTTPBearer</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/users/me/consent/{channel}</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Revoke Consent</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2700,7 +2704,7 @@
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -2712,17 +2716,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/users/{user_id}</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>Get Profile</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2745,12 +2749,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2778,12 +2782,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/users/{user_id}/follow-status</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>Status Endpoint</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2811,28 +2815,28 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/{user_id}/followers</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Followers</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2844,17 +2848,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>/health/circuit-breakers</t>
+          <t>/api/v1/users/{user_id}/following</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Circuit-breaker snapshot (admin-only)</t>
+          <t>Following</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -2865,7 +2869,7 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -2877,12 +2881,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/health</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Liveness probe</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2910,12 +2914,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/health/circuit-breakers</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Circuit-breaker snapshot (admin-only)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2925,7 +2929,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>HTTPBearer</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -2943,12 +2947,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/health/db</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>Database readiness probe</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2963,6 +2967,72 @@
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2979,7 +3049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3291,7 +3361,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FollowCounts</t>
+          <t>FlagList</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3301,14 +3371,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>followers, following</t>
+          <t>flags</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FollowListPage</t>
+          <t>FlagOverride</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3318,14 +3388,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>user_id, enabled</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FollowStatus</t>
+          <t>FlagOverrideResponse</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3335,14 +3405,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
+          <t>flag, user_id, action</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FollowUserView</t>
+          <t>FlagView</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3352,14 +3422,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url, followed_at</t>
+          <t>name, env_value, builtin_value, overridden_user_count</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>GroupRoomCreate</t>
+          <t>FollowCounts</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3369,14 +3439,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>title, member_ids</t>
+          <t>followers, following</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HTTPValidationError</t>
+          <t>FollowListPage</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3386,14 +3456,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HomeFeedPage</t>
+          <t>FollowStatus</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3403,14 +3473,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>items, next_cursor, cache_hit</t>
+          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LikeUser</t>
+          <t>FollowUserView</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3420,14 +3490,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url</t>
+          <t>user_id, display_name, avatar_url, followed_at</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LikeUserPage</t>
+          <t>GroupRoomCreate</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3437,14 +3507,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>title, member_ids</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>HTTPValidationError</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3454,14 +3524,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>detail</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LoginResponse</t>
+          <t>HomeFeedPage</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3471,14 +3541,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MarkReadResponse</t>
+          <t>LikeUser</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3488,14 +3558,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>updated</t>
+          <t>user_id, display_name, avatar_url</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MediaView</t>
+          <t>LikeUserPage</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3505,14 +3575,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MemberReadState</t>
+          <t>LoginRequest</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3522,14 +3592,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>user_id, last_read_message_id</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MessageCreate</t>
+          <t>LoginResponse</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3539,14 +3609,14 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>body, media_id</t>
+          <t>user, tokens</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MessagePage</t>
+          <t>MarkReadResponse</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3556,14 +3626,14 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>updated</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MessageView</t>
+          <t>MediaView</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3573,14 +3643,14 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>id, room_id, sender_id, body, media_id, created_at, is_edited</t>
+          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>NotificationPage</t>
+          <t>MemberReadState</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3590,14 +3660,14 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>user_id, last_read_message_id</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>NotificationView</t>
+          <t>MessageCreate</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3607,14 +3677,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
+          <t>body, media_id</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PostCreate</t>
+          <t>MessagePage</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3624,14 +3694,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>body, visibility</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PostPage</t>
+          <t>MessageView</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3641,14 +3711,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>id, room_id, sender_id, body, media_id, created_at, is_edited</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PostUpdate</t>
+          <t>NotificationPage</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3658,14 +3728,14 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>body, visibility, version</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PostView</t>
+          <t>NotificationView</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3675,14 +3745,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited</t>
+          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>PresenceView</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3692,14 +3762,14 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>user_id, online, connections</t>
+          <t>body, visibility</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>PostPage</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3709,14 +3779,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>PostUpdate</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3726,14 +3796,14 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>body, visibility, version</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>PostView</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3743,14 +3813,14 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ReadReceiptsList</t>
+          <t>PresenceView</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3760,14 +3830,14 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>members</t>
+          <t>user_id, online, connections</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ReadRequest</t>
+          <t>ProfilePublic</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3777,14 +3847,14 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>message_id</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>ProfileSelf</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3794,14 +3864,14 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3811,14 +3881,14 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>ReadReceiptsList</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3828,14 +3898,14 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>members</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ReportCreate</t>
+          <t>ReadRequest</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3845,14 +3915,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>target_type, target_id, reason, details</t>
+          <t>message_id</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ReportPage</t>
+          <t>RefreshRequest</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3862,27 +3932,31 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>refresh_token</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ReportStatus</t>
+          <t>RegisterRequest</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr"/>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>email, password</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ReportUpdate</t>
+          <t>RegisterResponse</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3892,14 +3966,14 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>status, resolution_note, version</t>
+          <t>user, message</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ReportView</t>
+          <t>ReportCreate</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3909,14 +3983,14 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>id, reporter_id, target_type, target_id, reason, details, status, reviewer_id, resolution_note, resolved_at, created_at, updated_at</t>
+          <t>target_type, target_id, reason, details</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>RoomMemberView</t>
+          <t>ReportPage</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3926,31 +4000,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>user_id, role, joined_at</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>RoomMembersList</t>
+          <t>ReportStatus</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>members</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>RoomUpdate</t>
+          <t>ReportUpdate</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3960,14 +4030,14 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>title, version</t>
+          <t>status, resolution_note, version</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>RoomView</t>
+          <t>ReportView</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3977,14 +4047,14 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>id, type, title, created_at, updated_at</t>
+          <t>id, reporter_id, target_type, target_id, reason, details, status, reviewer_id, resolution_note, resolved_at, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>UnreadCount</t>
+          <t>RoomMemberView</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3994,14 +4064,14 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>unread</t>
+          <t>user_id, role, joined_at</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>RoomMembersList</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4011,22 +4081,90 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>members</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>RoomUpdate</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>title, version</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>RoomView</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>id, type, title, created_at, updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>UnreadCount</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>unread</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t>ValidationError</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
contract export finalization (5 artifacts + enriched docs + drift on all)
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -47,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,41 +418,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Path</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Auth</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Rate Limit</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Errors</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Request Schema</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Response Codes</t>
         </is>
@@ -477,11 +502,21 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -510,11 +545,21 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -548,10 +593,20 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>LoginRequest</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -580,11 +635,21 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
         <is>
           <t>204</t>
         </is>
@@ -613,11 +678,21 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -651,10 +726,20 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>RefreshRequest</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -688,10 +773,20 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>RegisterRequest</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>201, 422</t>
         </is>
@@ -720,11 +815,21 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -753,11 +858,21 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -786,11 +901,21 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -819,11 +944,21 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -852,15 +987,25 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>DirectRoomCreate</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -889,15 +1034,25 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>GroupRoomCreate</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>201, 422</t>
         </is>
@@ -926,11 +1081,21 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -959,15 +1124,25 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>RoomUpdate</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -996,11 +1171,21 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1029,15 +1214,25 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>AddMemberRequest</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>201, 422</t>
         </is>
@@ -1066,11 +1261,21 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -1099,11 +1304,21 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1132,15 +1347,25 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>MessageCreate</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>201, 422</t>
         </is>
@@ -1169,15 +1394,25 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
           <t>ReadRequest</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1206,11 +1441,21 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1239,11 +1484,21 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -1272,11 +1527,21 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1305,11 +1570,21 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -1338,15 +1613,25 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
           <t>CommentUpdate</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1375,11 +1660,21 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1408,11 +1703,21 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1441,11 +1746,21 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -1474,15 +1789,25 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>FlagOverride</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1511,11 +1836,21 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -1544,11 +1879,21 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -1577,11 +1922,21 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -1610,11 +1965,21 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -1643,11 +2008,21 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -1676,11 +2051,21 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -1709,11 +2094,21 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -1742,11 +2137,21 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1775,15 +2180,25 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
           <t>Body_upload_media_api_v1_media_post</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>201, 422</t>
         </is>
@@ -1812,11 +2227,21 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -1845,11 +2270,21 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1878,11 +2313,21 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1911,11 +2356,21 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G44" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -1944,15 +2399,25 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
           <t>ReportCreate</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>201, 422</t>
         </is>
@@ -1981,15 +2446,25 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
           <t>ReportUpdate</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2018,11 +2493,21 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G47" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -2051,11 +2536,21 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G48" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -2084,11 +2579,21 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2117,11 +2622,21 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2150,11 +2665,21 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2183,11 +2708,21 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G52" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -2216,11 +2751,21 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G53" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2249,15 +2794,25 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
           <t>PostCreate</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>201, 422</t>
         </is>
@@ -2286,11 +2841,21 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G55" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2319,11 +2884,21 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G56" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -2352,11 +2927,21 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2385,15 +2970,25 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
           <t>PostUpdate</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2422,11 +3017,21 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2455,15 +3060,25 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
           <t>CommentCreate</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
+      <c r="I60" t="inlineStr">
         <is>
           <t>201, 422</t>
         </is>
@@ -2492,11 +3107,21 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G61" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2525,11 +3150,21 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G62" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2558,11 +3193,21 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G63" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2591,15 +3236,25 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
           <t>ProfileUpdate</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
+      <c r="I64" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2628,11 +3283,21 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G65" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2661,15 +3326,25 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
           <t>ConsentGrantRequest</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="I66" t="inlineStr">
         <is>
           <t>201, 422</t>
         </is>
@@ -2698,11 +3373,21 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G67" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
         <is>
           <t>204, 422</t>
         </is>
@@ -2731,11 +3416,21 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G68" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2764,11 +3459,21 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G69" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2797,11 +3502,21 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G70" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2830,11 +3545,21 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G71" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2863,11 +3588,21 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
         <is>
           <t>200, 422</t>
         </is>
@@ -2899,8 +3634,18 @@
           <t>public</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G73" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2929,11 +3674,21 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>HTTPBearer</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr"/>
+          <t>authenticated</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2965,8 +3720,18 @@
           <t>public</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -2998,8 +3763,18 @@
           <t>public</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G76" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -3031,8 +3806,18 @@
           <t>public</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="G77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -3049,21 +3834,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:D66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Properties</t>
         </is>
@@ -3085,6 +3881,11 @@
           <t>user_id</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3102,6 +3903,11 @@
           <t>id, actor_id, action, entity, entity_id, before, after, ip, user_agent, request_id, created_at</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>id, actor_id, action, entity, entity_id, before, after, ip, user_agent, request_id, created_at</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3116,6 +3922,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>items, next_cursor</t>
         </is>
       </c>
@@ -3133,6 +3944,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>access_token, refresh_token, expires_in</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>access_token, refresh_token, token_type, expires_in</t>
         </is>
       </c>
@@ -3153,6 +3969,11 @@
           <t>file</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>file</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3170,6 +3991,11 @@
           <t>message</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3184,6 +4010,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>body</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>body, parent_id</t>
         </is>
       </c>
@@ -3201,6 +4032,11 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>items, next_cursor</t>
         </is>
       </c>
@@ -3221,6 +4057,11 @@
           <t>body, version</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>body, version</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3235,6 +4076,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at, is_liked_by_me, is_edited, replies</t>
         </is>
       </c>
@@ -3255,6 +4101,11 @@
           <t>channel</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>channel</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3272,6 +4123,11 @@
           <t>consents</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>consents</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3289,6 +4145,11 @@
           <t>channel, granted, granted_at, revoked_at</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>channel, granted, granted_at, revoked_at</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3306,6 +4167,11 @@
           <t>message, hard_delete_after</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>message, hard_delete_after</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3323,6 +4189,11 @@
           <t>scheduled, scheduled_hard_delete_at, status</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>scheduled, scheduled_hard_delete_at, status</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3340,6 +4211,11 @@
           <t>other_user_id</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>other_user_id</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3354,6 +4230,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
@@ -3374,6 +4255,11 @@
           <t>flags</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>flags</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3391,6 +4277,11 @@
           <t>user_id, enabled</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>user_id, enabled</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3405,7 +4296,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>flag, user_id, action</t>
+          <t>flag, user_id, enabled, action</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>flag, user_id, enabled, action</t>
         </is>
       </c>
     </row>
@@ -3422,7 +4318,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>name, env_value, builtin_value, overridden_user_count</t>
+          <t>name, env_value, builtin_value</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>name, env_value, builtin_value</t>
         </is>
       </c>
     </row>
@@ -3442,6 +4343,11 @@
           <t>followers, following</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>followers, following</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3456,6 +4362,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>items, next_cursor</t>
         </is>
       </c>
@@ -3476,6 +4387,11 @@
           <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3490,6 +4406,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>user_id, followed_at</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
           <t>user_id, display_name, avatar_url, followed_at</t>
         </is>
       </c>
@@ -3507,6 +4428,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>title, member_ids</t>
         </is>
       </c>
@@ -3522,7 +4448,8 @@
           <t>object</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
         <is>
           <t>detail</t>
         </is>
@@ -3541,6 +4468,11 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
@@ -3558,6 +4490,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
           <t>user_id, display_name, avatar_url</t>
         </is>
       </c>
@@ -3575,6 +4512,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
           <t>items, next_cursor</t>
         </is>
       </c>
@@ -3595,6 +4537,11 @@
           <t>email, password</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>email, password</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3612,6 +4559,11 @@
           <t>user, tokens</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>user, tokens</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3629,6 +4581,11 @@
           <t>updated</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>updated</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3646,6 +4603,11 @@
           <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3663,6 +4625,11 @@
           <t>user_id, last_read_message_id</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>user_id, last_read_message_id</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3677,6 +4644,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
+          <t>body</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
           <t>body, media_id</t>
         </is>
       </c>
@@ -3694,6 +4666,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>items, next_cursor</t>
         </is>
       </c>
@@ -3711,6 +4688,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
+          <t>id, room_id, sender_id, body, media_id, created_at</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
           <t>id, room_id, sender_id, body, media_id, created_at, is_edited</t>
         </is>
       </c>
@@ -3728,6 +4710,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
           <t>items, next_cursor</t>
         </is>
       </c>
@@ -3748,6 +4735,11 @@
           <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3762,6 +4754,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
+          <t>body</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
           <t>body, visibility</t>
         </is>
       </c>
@@ -3779,6 +4776,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
           <t>items, next_cursor</t>
         </is>
       </c>
@@ -3796,6 +4798,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
           <t>body, visibility, version</t>
         </is>
       </c>
@@ -3813,6 +4820,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
           <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited</t>
         </is>
       </c>
@@ -3833,6 +4845,11 @@
           <t>user_id, online, connections</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>user_id, online, connections</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3847,6 +4864,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
+          <t>user_id, visibility</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
           <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
@@ -3864,6 +4886,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
+          <t>user_id, visibility, pii_visibility, version, created_at, updated_at</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
           <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
@@ -3881,6 +4908,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
           <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
@@ -3901,6 +4933,11 @@
           <t>members</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>members</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3918,6 +4955,11 @@
           <t>message_id</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>message_id</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3935,6 +4977,11 @@
           <t>refresh_token</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>refresh_token</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3952,6 +4999,11 @@
           <t>email, password</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>email, password</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3969,6 +5021,11 @@
           <t>user, message</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>user, message</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3983,6 +5040,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
+          <t>target_type, target_id, reason</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
           <t>target_type, target_id, reason, details</t>
         </is>
       </c>
@@ -4000,6 +5062,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
           <t>items, next_cursor</t>
         </is>
       </c>
@@ -4016,6 +5083,7 @@
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4030,6 +5098,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
+          <t>status, version</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
           <t>status, resolution_note, version</t>
         </is>
       </c>
@@ -4050,6 +5123,11 @@
           <t>id, reporter_id, target_type, target_id, reason, details, status, reviewer_id, resolution_note, resolved_at, created_at, updated_at</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>id, reporter_id, target_type, target_id, reason, details, status, reviewer_id, resolution_note, resolved_at, created_at, updated_at</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4067,6 +5145,11 @@
           <t>user_id, role, joined_at</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>user_id, role, joined_at</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4084,6 +5167,11 @@
           <t>members</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>members</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4101,6 +5189,11 @@
           <t>title, version</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>title, version</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4118,6 +5211,11 @@
           <t>id, type, title, created_at, updated_at</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>id, type, title, created_at, updated_at</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4135,6 +5233,11 @@
           <t>unread</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>unread</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4152,6 +5255,11 @@
           <t>id, role, is_active, is_verified, created_at</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4165,6 +5273,11 @@
         </is>
       </c>
       <c r="C66" t="inlineStr">
+        <is>
+          <t>loc, msg, type</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
         <is>
           <t>loc, msg, type, input, ctx</t>
         </is>

</xml_diff>

<commit_message>
chore(contracts): regenerate for /api/v1/search; pin types.ts generator
</commit_message>
<xml_diff>
--- a/contracts/api_reference.xlsx
+++ b/contracts/api_reference.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -573,12 +573,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>/api/v1/auth/forgot-password</t>
+          <t>/api/v1/auth/change-password</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Forgot Password</t>
+          <t>Change Password</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -588,7 +588,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>ForgotPasswordRequest</t>
+          <t>ChangePasswordRequest</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -620,12 +620,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>/api/v1/auth/login</t>
+          <t>/api/v1/auth/forgot-password</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Forgot Password</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>ForgotPasswordRequest</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -667,12 +667,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>/api/v1/auth/logout</t>
+          <t>/api/v1/auth/login</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Logout</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>authenticated</t>
+          <t>public</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -692,30 +692,34 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>LoginRequest</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>/api/v1/auth/me</t>
+          <t>/api/v1/auth/logout</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Me</t>
+          <t>Logout</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -741,24 +745,24 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>/api/v1/auth/refresh</t>
+          <t>/api/v1/auth/me</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Refresh</t>
+          <t>Me</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -768,7 +772,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -778,17 +782,13 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>422</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>RefreshRequest</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -800,12 +800,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/api/v1/auth/register</t>
+          <t>/api/v1/auth/refresh</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Register</t>
+          <t>Refresh</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -830,12 +830,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>RefreshRequest</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -847,12 +847,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>/api/v1/auth/reset-password</t>
+          <t>/api/v1/auth/register</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Reset Password</t>
+          <t>Register</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -877,12 +877,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ResetPasswordRequest</t>
+          <t>RegisterRequest</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
@@ -894,12 +894,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>/api/v1/auth/verify-email</t>
+          <t>/api/v1/auth/reset-password</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Verify Email</t>
+          <t>Reset Password</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>VerifyEmailRequest</t>
+          <t>ResetPasswordRequest</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -936,27 +936,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>/api/v1/blocks/{user_id}</t>
+          <t>/api/v1/auth/verify-email</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Unblock</t>
+          <t>Verify Email</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>auth</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>authenticated</t>
+          <t>public</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -969,17 +969,21 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>VerifyEmailRequest</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -989,7 +993,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Block</t>
+          <t>Unblock</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1022,22 +1026,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/api/v1/chat/messages/{message_id}</t>
+          <t>/api/v1/blocks/{user_id}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Delete Message</t>
+          <t>Block</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>chat</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1065,17 +1069,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms</t>
+          <t>/api/v1/chat/messages/{message_id}</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>List My Rooms</t>
+          <t>Delete Message</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1095,30 +1099,30 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>422</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/direct</t>
+          <t>/api/v1/chat/rooms</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Create Direct Room</t>
+          <t>List My Rooms</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1138,17 +1142,13 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>422</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>DirectRoomCreate</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -1160,12 +1160,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/group</t>
+          <t>/api/v1/chat/rooms/direct</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Create Group</t>
+          <t>Create Direct Room</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1190,29 +1190,29 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>GroupRoomCreate</t>
+          <t>DirectRoomCreate</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}</t>
+          <t>/api/v1/chat/rooms/group</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Get Room</t>
+          <t>Create Group</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1235,17 +1235,21 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>GroupRoomCreate</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1255,7 +1259,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Update Room</t>
+          <t>Get Room</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1278,11 +1282,7 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>RoomUpdate</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1292,17 +1292,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/members</t>
+          <t>/api/v1/chat/rooms/{room_id}</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>List Members</t>
+          <t>Update Room</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1325,7 +1325,11 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>RoomUpdate</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1335,7 +1339,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1345,7 +1349,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Add Member</t>
+          <t>List Members</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1368,31 +1372,27 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>AddMemberRequest</t>
-        </is>
-      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/members/{target_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/members</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Remove Member</t>
+          <t>Add Member</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1415,27 +1415,31 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>AddMemberRequest</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/messages</t>
+          <t>/api/v1/chat/rooms/{room_id}/members/{target_id}</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>List Messages</t>
+          <t>Remove Member</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1461,14 +1465,14 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1478,7 +1482,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Send Message</t>
+          <t>List Messages</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1501,14 +1505,10 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>MessageCreate</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -1520,12 +1520,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/read</t>
+          <t>/api/v1/chat/rooms/{room_id}/messages</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mark Read</t>
+          <t>Send Message</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1550,29 +1550,29 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>ReadRequest</t>
+          <t>MessageCreate</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/read-receipts</t>
+          <t>/api/v1/chat/rooms/{room_id}/read</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>List Read Receipts</t>
+          <t>Mark Read</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1595,7 +1595,11 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>ReadRequest</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1605,17 +1609,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/typing</t>
+          <t>/api/v1/chat/rooms/{room_id}/read-receipts</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Typing</t>
+          <t>List Read Receipts</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1641,24 +1645,24 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>/api/v1/chat/rooms/{room_id}/unread-count</t>
+          <t>/api/v1/chat/rooms/{room_id}/typing</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Unread Count</t>
+          <t>Typing</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1684,29 +1688,29 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>/api/v1/comments/{comment_id}</t>
+          <t>/api/v1/chat/rooms/{room_id}/unread-count</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Delete Comment</t>
+          <t>Unread Count</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>chat</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1727,14 +1731,14 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1744,7 +1748,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Update Comment</t>
+          <t>Delete Comment</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1767,36 +1771,32 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>CommentUpdate</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>/api/v1/feed/explore</t>
+          <t>/api/v1/comments/{comment_id}</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Explore Feed</t>
+          <t>Update Comment</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>feed</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1814,7 +1814,11 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>CommentUpdate</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -1829,12 +1833,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>/api/v1/feed/home</t>
+          <t>/api/v1/feed/explore</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Home Feed</t>
+          <t>Explore Feed</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1872,17 +1876,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>/api/v1/flags</t>
+          <t>/api/v1/feed/home</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>List Flags</t>
+          <t>Home Feed</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>flags</t>
+          <t>feed</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1897,30 +1901,30 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>422</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>/api/v1/flags/{flag_name}/override</t>
+          <t>/api/v1/flags</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Override Flag</t>
+          <t>List Flags</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1940,39 +1944,35 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>422</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>FlagOverride</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/api/v1/follows/{user_id}</t>
+          <t>/api/v1/flags/{flag_name}/override</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Unfollow a user (idempotent)</t>
+          <t>Override Flag</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>flags</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1990,17 +1990,21 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>FlagOverride</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2010,7 +2014,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Follow a user (idempotent)</t>
+          <t>Unfollow a user (idempotent)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2048,17 +2052,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/api/v1/gdpr/cancel-delete</t>
+          <t>/api/v1/follows/{user_id}</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Cancel Deletion</t>
+          <t>Follow a user (idempotent)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>gdpr</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2073,30 +2077,30 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>422</t>
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/api/v1/gdpr/deletion-status</t>
+          <t>/api/v1/gdpr/cancel-delete</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Deletion Status</t>
+          <t>Cancel Deletion</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2134,12 +2138,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/api/v1/gdpr/export</t>
+          <t>/api/v1/gdpr/deletion-status</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Export Data</t>
+          <t>Deletion Status</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2172,22 +2176,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}</t>
+          <t>/api/v1/gdpr/export</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Unlike</t>
+          <t>Export Data</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>likes</t>
+          <t>gdpr</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2202,20 +2206,20 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2225,7 +2229,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Like</t>
+          <t>Unlike</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2258,17 +2262,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
+          <t>/api/v1/likes/{target_type}/{target_id}</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>List Likers</t>
+          <t>Like</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2294,29 +2298,29 @@
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/api/v1/media</t>
+          <t>/api/v1/likes/{target_type}/{target_id}/users</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Upload Media</t>
+          <t>List Likers</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>likes</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2334,31 +2338,27 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Body_upload_media_api_v1_media_post</t>
-        </is>
-      </c>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}</t>
+          <t>/api/v1/media</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Delete Media</t>
+          <t>Upload Media</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2381,17 +2381,21 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Body_upload_media_api_v1_media_post</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2401,7 +2405,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Get Media</t>
+          <t>Delete Media</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2427,24 +2431,24 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
+          <t>/api/v1/media/{media_id}</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Attach To Post</t>
+          <t>Get Media</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2482,12 +2486,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>/api/v1/media/{media_id}/avatar</t>
+          <t>/api/v1/media/{media_id}/attach/{post_id}</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Set Avatar</t>
+          <t>Attach To Post</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2520,22 +2524,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>/api/v1/moderation/reports</t>
+          <t>/api/v1/media/{media_id}/avatar</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>List Reports</t>
+          <t>Set Avatar</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>moderation</t>
+          <t>media</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2563,7 +2567,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2573,7 +2577,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Create Report</t>
+          <t>List Reports</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2596,31 +2600,27 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>ReportCreate</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>/api/v1/moderation/reports/{report_id}</t>
+          <t>/api/v1/moderation/reports</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Update Report</t>
+          <t>Create Report</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2645,34 +2645,34 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>ReportUpdate</t>
+          <t>ReportCreate</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>/api/v1/mutes/{user_id}</t>
+          <t>/api/v1/moderation/reports/{report_id}</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Unmute</t>
+          <t>Update Report</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>moderation</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2690,17 +2690,21 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>ReportUpdate</t>
+        </is>
+      </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2710,7 +2714,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Mute</t>
+          <t>Unmute</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2743,22 +2747,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>/api/v1/notifications</t>
+          <t>/api/v1/mutes/{user_id}</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>List Notifications</t>
+          <t>Mute</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>notifications</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2779,24 +2783,24 @@
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/read-all</t>
+          <t>/api/v1/notifications</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Mark All Read</t>
+          <t>List Notifications</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2816,30 +2820,30 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>422</t>
         </is>
       </c>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/unread-count</t>
+          <t>/api/v1/notifications/read-all</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Unread Count</t>
+          <t>Mark All Read</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2872,17 +2876,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}</t>
+          <t>/api/v1/notifications/unread-count</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Delete Notification</t>
+          <t>Unread Count</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2902,30 +2906,30 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>/api/v1/notifications/{notif_id}/read</t>
+          <t>/api/v1/notifications/{notif_id}</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Mark Read</t>
+          <t>Delete Notification</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2951,7 +2955,7 @@
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -2963,17 +2967,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>/api/v1/posts</t>
+          <t>/api/v1/notifications/{notif_id}/read</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Create Post</t>
+          <t>Mark Read</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>posts</t>
+          <t>notifications</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2991,31 +2995,27 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>PostCreate</t>
-        </is>
-      </c>
+      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>/api/v1/posts/by-author/{author_id}</t>
+          <t>/api/v1/posts</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>List By Author</t>
+          <t>Create Post</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3038,27 +3038,31 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>PostCreate</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}</t>
+          <t>/api/v1/posts/by-author/{author_id}</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Delete Post</t>
+          <t>List By Author</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3084,14 +3088,14 @@
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3101,7 +3105,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Get Post</t>
+          <t>Delete Post</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3127,14 +3131,14 @@
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3144,7 +3148,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Update Post</t>
+          <t>Get Post</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3167,11 +3171,7 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>PostUpdate</t>
-        </is>
-      </c>
+      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -3181,22 +3181,22 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>/api/v1/posts/{post_id}/comments</t>
+          <t>/api/v1/posts/{post_id}</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>List Comments</t>
+          <t>Update Post</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>posts</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3214,7 +3214,11 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>PostUpdate</t>
+        </is>
+      </c>
       <c r="I63" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -3224,7 +3228,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3234,7 +3238,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Create Comment</t>
+          <t>List Comments</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3257,36 +3261,32 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>CommentCreate</t>
-        </is>
-      </c>
+      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>/api/v1/presence/{user_id}</t>
+          <t>/api/v1/posts/{post_id}/comments</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Get Presence</t>
+          <t>Create Comment</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>presence</t>
+          <t>comments</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3304,32 +3304,36 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>CommentCreate</t>
+        </is>
+      </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/presence/{user_id}</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Delete Me</t>
+          <t>Get Presence</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>presence</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3344,13 +3348,13 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>422</t>
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -3362,17 +3366,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/search</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Get Me</t>
+          <t>Search</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>search</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3387,30 +3391,30 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>422</t>
         </is>
       </c>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>PATCH</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>/api/v1/users/me</t>
+          <t>/api/v1/users</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Update Me</t>
+          <t>List Users</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3433,11 +3437,7 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>ProfileUpdate</t>
-        </is>
-      </c>
+      <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
         <is>
           <t>200, 422</t>
@@ -3447,17 +3447,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>List Consents</t>
+          <t>Delete Me</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3490,17 +3490,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Grant Consent</t>
+          <t>Get Me</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3520,34 +3520,30 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>422</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>ConsentGrantRequest</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr">
         <is>
-          <t>201, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>/api/v1/users/me/consent/{channel}</t>
+          <t>/api/v1/users/me</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Revoke Consent</t>
+          <t>Update Me</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3570,10 +3566,14 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>ProfileUpdate</t>
+        </is>
+      </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>204, 422</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -3585,12 +3585,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Get Profile</t>
+          <t>List Consents</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3610,35 +3610,35 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>422</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-counts</t>
+          <t>/api/v1/users/me/consent</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Counts</t>
+          <t>Grant Consent</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3656,32 +3656,36 @@
           <t>422</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>ConsentGrantRequest</t>
+        </is>
+      </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>201, 422</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/follow-status</t>
+          <t>/api/v1/users/me/consent/{channel}</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Status Endpoint</t>
+          <t>Revoke Consent</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3702,7 +3706,7 @@
       <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr">
         <is>
-          <t>200, 422</t>
+          <t>204, 422</t>
         </is>
       </c>
     </row>
@@ -3714,17 +3718,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/followers</t>
+          <t>/api/v1/users/{user_id}</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Followers</t>
+          <t>Get Profile</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>follows</t>
+          <t>users</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3757,12 +3761,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>/api/v1/users/{user_id}/following</t>
+          <t>/api/v1/users/{user_id}/follow-counts</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Following</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3800,22 +3804,22 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>/health</t>
+          <t>/api/v1/users/{user_id}/follow-status</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Liveness probe</t>
+          <t>Status Endpoint</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3825,13 +3829,13 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>422</t>
         </is>
       </c>
       <c r="H77" t="inlineStr"/>
       <c r="I77" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -3843,17 +3847,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>/health/circuit-breakers</t>
+          <t>/api/v1/users/{user_id}/followers</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Circuit-breaker snapshot (admin-only)</t>
+          <t>Followers</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3868,13 +3872,13 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>422</t>
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -3886,22 +3890,22 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>/health/db</t>
+          <t>/api/v1/users/{user_id}/following</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Database readiness probe</t>
+          <t>Following</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>follows</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3911,13 +3915,13 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>422</t>
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
       <c r="I79" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>200, 422</t>
         </is>
       </c>
     </row>
@@ -3929,12 +3933,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>/health/ready</t>
+          <t>/health</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Readiness probe (aggregate)</t>
+          <t>Liveness probe</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3972,12 +3976,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>/health/redis</t>
+          <t>/health/circuit-breakers</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Redis readiness probe</t>
+          <t>Circuit-breaker snapshot (admin-only)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3987,7 +3991,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>public</t>
+          <t>authenticated</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4002,6 +4006,135 @@
       </c>
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>/health/db</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Database readiness probe</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>/health/ready</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Readiness probe (aggregate)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>/health/redis</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Redis readiness probe</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>health</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -4018,7 +4151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4074,7 +4207,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AuditLogView</t>
+          <t>AdminUserPage</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4084,19 +4217,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>id, actor_id, action, entity, entity_id, before, after, ip, user_agent, request_id, created_at</t>
+          <t>items</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>id, actor_id, action, entity, entity_id, before, after, ip, user_agent, request_id, created_at</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AuditPage</t>
+          <t>AdminUserView</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4106,19 +4239,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>items</t>
+          <t>id, role, is_active, is_verified, created_at</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>id, role, is_active, is_verified, created_at, display_name, avatar_url</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AuthTokens</t>
+          <t>AuditLogView</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4128,19 +4261,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>access_token, refresh_token, expires_in</t>
+          <t>id, actor_id, action, entity, entity_id, before, after, ip, user_agent, request_id, created_at</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>access_token, refresh_token, token_type, expires_in</t>
+          <t>id, actor_id, action, entity, entity_id, before, after, ip, user_agent, request_id, created_at</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Body_upload_media_api_v1_media_post</t>
+          <t>AuditPage</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4150,19 +4283,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>items</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CancelResponse</t>
+          <t>AuthTokens</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4172,19 +4305,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>access_token, refresh_token, expires_in</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>access_token, refresh_token, token_type, expires_in</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CommentCreate</t>
+          <t>Body_upload_media_api_v1_media_post</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4194,19 +4327,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>body</t>
+          <t>file</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>body, parent_id</t>
+          <t>file</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CommentPage</t>
+          <t>CancelResponse</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4216,19 +4349,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>items</t>
+          <t>message</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>message</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CommentUpdate</t>
+          <t>ChangePasswordRequest</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4238,19 +4371,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>body, version</t>
+          <t>current_password, new_password</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>body, version</t>
+          <t>current_password, new_password</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CommentView</t>
+          <t>CommentCreate</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4260,19 +4393,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at</t>
+          <t>body</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at, is_liked_by_me, is_edited, replies</t>
+          <t>body, parent_id</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ConsentGrantRequest</t>
+          <t>CommentPage</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4282,19 +4415,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>items</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ConsentList</t>
+          <t>CommentUpdate</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4304,19 +4437,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>consents</t>
+          <t>body, version</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>consents</t>
+          <t>body, version</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ConsentRecord</t>
+          <t>CommentView</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4326,19 +4459,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>channel, granted, granted_at, revoked_at</t>
+          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>channel, granted, granted_at, revoked_at</t>
+          <t>id, post_id, author_id, parent_id, depth, body, like_count, created_at, updated_at, is_liked_by_me, is_edited, replies</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DeleteMeResponse</t>
+          <t>ConsentGrantRequest</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4348,19 +4481,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>message, hard_delete_after</t>
+          <t>channel</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>message, hard_delete_after</t>
+          <t>channel</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DeletionStatusView</t>
+          <t>ConsentList</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -4370,19 +4503,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>scheduled, scheduled_hard_delete_at, status</t>
+          <t>consents</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>scheduled, scheduled_hard_delete_at, status</t>
+          <t>consents</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DirectRoomCreate</t>
+          <t>ConsentRecord</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -4392,19 +4525,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>other_user_id</t>
+          <t>channel, granted, granted_at, revoked_at</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>other_user_id</t>
+          <t>channel, granted, granted_at, revoked_at</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ExploreFeedPage</t>
+          <t>DeleteMeResponse</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -4414,19 +4547,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>items</t>
+          <t>message, hard_delete_after</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>items, next_cursor, cache_hit</t>
+          <t>message, hard_delete_after</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FlagList</t>
+          <t>DeletionStatusView</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -4436,19 +4569,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>flags</t>
+          <t>scheduled, scheduled_hard_delete_at, status</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>flags</t>
+          <t>scheduled, scheduled_hard_delete_at, status</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FlagOverride</t>
+          <t>DirectRoomCreate</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4458,19 +4591,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>user_id, enabled</t>
+          <t>other_user_id</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>user_id, enabled</t>
+          <t>other_user_id</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FlagOverrideResponse</t>
+          <t>ExploreFeedPage</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -4480,19 +4613,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>flag, user_id, enabled, action</t>
+          <t>items</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>flag, user_id, enabled, action</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FlagView</t>
+          <t>FlagList</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4502,19 +4635,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>name, env_value, builtin_value</t>
+          <t>flags</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>name, env_value, builtin_value</t>
+          <t>flags</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FollowCounts</t>
+          <t>FlagOverride</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4524,19 +4657,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>followers, following</t>
+          <t>user_id, enabled</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>followers, following</t>
+          <t>user_id, enabled</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FollowListPage</t>
+          <t>FlagOverrideResponse</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4546,19 +4679,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>items</t>
+          <t>flag, user_id, enabled, action</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>flag, user_id, enabled, action</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FollowStatus</t>
+          <t>FlagView</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4568,19 +4701,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
+          <t>name, env_value, builtin_value</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
+          <t>name, env_value, builtin_value</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FollowUserView</t>
+          <t>FollowCounts</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4590,19 +4723,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>user_id, followed_at</t>
+          <t>followers, following</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url, followed_at</t>
+          <t>followers, following</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ForgotPasswordRequest</t>
+          <t>FollowListPage</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4612,19 +4745,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>items</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GroupRoomCreate</t>
+          <t>FollowStatus</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4634,19 +4767,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>title, member_ids</t>
+          <t>is_following, is_followed_by, is_blocked_by_me, has_blocked_me, is_muted_by_me</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>HTTPValidationError</t>
+          <t>FollowUserView</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4654,17 +4787,21 @@
           <t>object</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>user_id, followed_at</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>user_id, display_name, avatar_url, followed_at</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>HomeFeedPage</t>
+          <t>ForgotPasswordRequest</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4674,19 +4811,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>items</t>
+          <t>email</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>items, next_cursor, cache_hit</t>
+          <t>email</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LikeUser</t>
+          <t>GroupRoomCreate</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4696,19 +4833,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>title</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>user_id, display_name, avatar_url</t>
+          <t>title, member_ids</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LikeUserPage</t>
+          <t>HTTPValidationError</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -4716,21 +4853,17 @@
           <t>object</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>items</t>
-        </is>
-      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>detail</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LoginRequest</t>
+          <t>HomeFeedPage</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -4740,19 +4873,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>items</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>items, next_cursor, cache_hit</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LoginResponse</t>
+          <t>LikeUser</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4762,19 +4895,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>user, tokens</t>
+          <t>user_id, display_name, avatar_url</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MarkReadResponse</t>
+          <t>LikeUserPage</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4784,19 +4917,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>updated</t>
+          <t>items</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>updated</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MediaView</t>
+          <t>LoginRequest</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4806,19 +4939,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
+          <t>email, password</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MemberReadState</t>
+          <t>LoginResponse</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4828,19 +4961,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>user_id, last_read_message_id</t>
+          <t>user, tokens</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>user_id, last_read_message_id</t>
+          <t>user, tokens</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MessageCreate</t>
+          <t>MarkReadResponse</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4850,19 +4983,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>body</t>
+          <t>updated</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>body, media_id</t>
+          <t>updated</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>MessagePage</t>
+          <t>MediaView</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4872,19 +5005,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>items</t>
+          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>id, owner_id, post_id, kind, mime, size_bytes, url, created_at</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MessageResponse</t>
+          <t>MemberReadState</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4894,19 +5027,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>user_id, last_read_message_id</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>message</t>
+          <t>user_id, last_read_message_id</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MessageView</t>
+          <t>MessageCreate</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4916,19 +5049,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>id, room_id, sender_id, body, media_id, created_at</t>
+          <t>body</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>id, room_id, sender_id, body, media_id, created_at, is_edited</t>
+          <t>body, media_id</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>NotificationPage</t>
+          <t>MessagePage</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4950,7 +5083,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>NotificationView</t>
+          <t>MessageResponse</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4960,19 +5093,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
+          <t>message</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
+          <t>message</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PostCreate</t>
+          <t>MessageView</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4982,19 +5115,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>body</t>
+          <t>id, room_id, sender_id, body, media_id, created_at</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>body, visibility</t>
+          <t>id, room_id, sender_id, body, media_id, created_at, is_edited</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>PostPage</t>
+          <t>NotificationPage</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5016,7 +5149,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PostUpdate</t>
+          <t>NotificationView</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5026,19 +5159,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>body, visibility, version</t>
+          <t>id, type, target_type, target_id, actor_id, is_read, read_at, preview, created_at</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PostView</t>
+          <t>PostCreate</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5048,19 +5181,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at</t>
+          <t>body</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited, media</t>
+          <t>body, visibility</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PresenceView</t>
+          <t>PostPage</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5070,19 +5203,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>user_id, online, connections</t>
+          <t>items</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>user_id, online, connections</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ProfilePublic</t>
+          <t>PostUpdate</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5092,19 +5225,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>user_id, visibility</t>
+          <t>version</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
+          <t>body, visibility, version</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ProfileSelf</t>
+          <t>PostView</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -5114,19 +5247,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>user_id, visibility, pii_visibility, version, created_at, updated_at</t>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
+          <t>id, author_id, body, visibility, like_count, comment_count, media_count, version, created_at, updated_at, is_liked_by_me, is_edited, media</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ProfileUpdate</t>
+          <t>PresenceView</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -5136,19 +5269,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>version</t>
+          <t>user_id, online, connections</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
+          <t>user_id, online, connections</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ReadReceiptsList</t>
+          <t>ProfilePublic</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -5158,19 +5291,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>members</t>
+          <t>user_id, visibility</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>members</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ReadRequest</t>
+          <t>ProfileSelf</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -5180,19 +5313,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>message_id</t>
+          <t>user_id, visibility, pii_visibility, version, created_at, updated_at</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>message_id</t>
+          <t>user_id, display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>RefreshRequest</t>
+          <t>ProfileUpdate</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -5202,19 +5335,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>version</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>refresh_token</t>
+          <t>display_name, bio, avatar_url, location, website, visibility, pii_visibility, dob, phone, address, version</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>RegisterRequest</t>
+          <t>ReadReceiptsList</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -5224,19 +5357,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>members</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>email, password</t>
+          <t>members</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>RegisterResponse</t>
+          <t>ReadRequest</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -5246,19 +5379,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>message_id</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>user, message</t>
+          <t>message_id</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ReportCreate</t>
+          <t>RefreshRequest</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -5268,19 +5401,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>target_type, target_id, reason</t>
+          <t>refresh_token</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>target_type, target_id, reason, details</t>
+          <t>refresh_token</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ReportPage</t>
+          <t>RegisterRequest</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -5290,33 +5423,41 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>items</t>
+          <t>email, password</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>items, next_cursor</t>
+          <t>email, password</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ReportStatus</t>
+          <t>RegisterResponse</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>user, message</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>user, message</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ReportUpdate</t>
+          <t>ReportCreate</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -5326,19 +5467,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>status, version</t>
+          <t>target_type, target_id, reason</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>status, resolution_note, version</t>
+          <t>target_type, target_id, reason, details</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ReportView</t>
+          <t>ReportPage</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -5348,41 +5489,33 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>id, reporter_id, target_type, target_id, reason, details, status, reviewer_id, resolution_note, resolved_at, created_at, updated_at, version</t>
+          <t>items</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>id, reporter_id, target_type, target_id, reason, details, status, reviewer_id, resolution_note, resolved_at, created_at, updated_at, version</t>
+          <t>items, next_cursor</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ResetPasswordRequest</t>
+          <t>ReportStatus</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>token, new_password</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>token, new_password</t>
-        </is>
-      </c>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>RoomMemberView</t>
+          <t>ReportUpdate</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -5392,19 +5525,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>user_id, role, joined_at</t>
+          <t>status, version</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>user_id, role, joined_at</t>
+          <t>status, resolution_note, version</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>RoomMembersList</t>
+          <t>ReportView</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -5414,19 +5547,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>members</t>
+          <t>id, reporter_id, target_type, target_id, reason, details, status, reviewer_id, resolution_note, resolved_at, created_at, updated_at, version</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>members</t>
+          <t>id, reporter_id, target_type, target_id, reason, details, status, reviewer_id, resolution_note, resolved_at, created_at, updated_at, version</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>RoomUpdate</t>
+          <t>ResetPasswordRequest</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -5436,19 +5569,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>title, version</t>
+          <t>token, new_password</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>title, version</t>
+          <t>token, new_password</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>RoomView</t>
+          <t>RoomMemberView</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -5458,19 +5591,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>id, type, title, created_at, updated_at</t>
+          <t>user_id, role, joined_at</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>id, type, title, created_at, updated_at</t>
+          <t>user_id, role, joined_at</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>UnreadCount</t>
+          <t>RoomMembersList</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -5480,19 +5613,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>unread</t>
+          <t>members</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>unread</t>
+          <t>members</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>UserPublic</t>
+          <t>RoomUpdate</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -5502,19 +5635,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>title, version</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>id, role, is_active, is_verified, created_at</t>
+          <t>title, version</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ValidationError</t>
+          <t>RoomView</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -5524,32 +5657,142 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>loc, msg, type</t>
+          <t>id, type, title, created_at, updated_at</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>loc, msg, type, input, ctx</t>
+          <t>id, type, title, created_at, updated_at</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
+          <t>SearchResults</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>query, users, posts</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>query, users, posts, next_cursor</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>SearchUserHit</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>user_id, display_name, avatar_url</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>UnreadCount</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>unread</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>unread</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>UserPublic</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>id, role, is_active, is_verified, created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ValidationError</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>loc, msg, type</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>loc, msg, type, input, ctx</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
           <t>VerifyEmailRequest</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>object</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
         <is>
           <t>token</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>token</t>
         </is>

</xml_diff>